<commit_message>
Update multiple Excel files with revised data for club ranges, club selector, clustered rounds, clutch score analysis, golf recommendations, and strokes gained summary.
</commit_message>
<xml_diff>
--- a/clustered_rounds.xlsx
+++ b/clustered_rounds.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N68"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1746,11 +1746,11 @@
         <v>-9.539999999999999</v>
       </c>
       <c r="M26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -1796,11 +1796,11 @@
         <v>-10.12</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -1846,11 +1846,11 @@
         <v>-10.12</v>
       </c>
       <c r="M28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -1896,11 +1896,11 @@
         <v>-9.960000000000001</v>
       </c>
       <c r="M29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -1946,11 +1946,11 @@
         <v>-10.96</v>
       </c>
       <c r="M30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -1996,11 +1996,11 @@
         <v>-5.1</v>
       </c>
       <c r="M31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2046,7 @@
         <v>-0.6</v>
       </c>
       <c r="M32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -2096,11 +2096,11 @@
         <v>-5.12</v>
       </c>
       <c r="M33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2146,11 +2146,11 @@
         <v>-11.7</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2196,11 +2196,11 @@
         <v>-6.38</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2246,11 +2246,11 @@
         <v>-8.119999999999999</v>
       </c>
       <c r="M36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2296,11 +2296,11 @@
         <v>-9.279999999999999</v>
       </c>
       <c r="M37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2346,11 +2346,11 @@
         <v>-10.28</v>
       </c>
       <c r="M38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2396,11 +2396,11 @@
         <v>-6.96</v>
       </c>
       <c r="M39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2446,11 +2446,11 @@
         <v>-7.28</v>
       </c>
       <c r="M40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2496,11 +2496,11 @@
         <v>-8.539999999999999</v>
       </c>
       <c r="M41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2546,11 +2546,11 @@
         <v>-8.960000000000001</v>
       </c>
       <c r="M42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2596,7 @@
         <v>-3.12</v>
       </c>
       <c r="M43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -2746,11 +2746,11 @@
         <v>-3.96</v>
       </c>
       <c r="M46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2796,7 @@
         <v>-1.28</v>
       </c>
       <c r="M47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
@@ -2846,11 +2846,11 @@
         <v>-1.7</v>
       </c>
       <c r="M48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2896,11 +2896,11 @@
         <v>-0.54</v>
       </c>
       <c r="M49" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2946,7 @@
         <v>-2.12</v>
       </c>
       <c r="M50" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
@@ -2996,7 +2996,7 @@
         <v>-4.12</v>
       </c>
       <c r="M51" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
@@ -3046,11 +3046,11 @@
         <v>-5.54</v>
       </c>
       <c r="M52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3096,7 @@
         <v>-2.12</v>
       </c>
       <c r="M53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
@@ -3146,7 +3146,7 @@
         <v>-1.7</v>
       </c>
       <c r="M54" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -3196,11 +3196,11 @@
         <v>-9.380000000000001</v>
       </c>
       <c r="M55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3246,7 @@
         <v>-3.7</v>
       </c>
       <c r="M56" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
@@ -3296,11 +3296,11 @@
         <v>-6.28</v>
       </c>
       <c r="M57" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3596,7 +3596,7 @@
         <v>-2.12</v>
       </c>
       <c r="M63" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
@@ -3646,11 +3646,11 @@
         <v>-3.12</v>
       </c>
       <c r="M64" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3696,7 +3696,7 @@
         <v>-4.7</v>
       </c>
       <c r="M65" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
@@ -3746,11 +3746,11 @@
         <v>-12.38</v>
       </c>
       <c r="M66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3796,11 +3796,11 @@
         <v>-4.12</v>
       </c>
       <c r="M67" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -3846,11 +3846,61 @@
         <v>-4.38</v>
       </c>
       <c r="M68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>All Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Bethpage Blue</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>34</v>
+      </c>
+      <c r="E69" t="n">
+        <v>8</v>
+      </c>
+      <c r="F69" t="n">
+        <v>5</v>
+      </c>
+      <c r="G69" t="n">
+        <v>1.889</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0.357</v>
+      </c>
+      <c r="J69" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="K69" t="n">
+        <v>-0.173</v>
+      </c>
+      <c r="L69" t="n">
+        <v>-5.44</v>
+      </c>
+      <c r="M69" t="n">
+        <v>3</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update multiple Excel files with revised data and change references in Golf Analytics notebook to the updated 'Golf Stats.xlsx'. Remove obsolete 'Copy of Golf Stats Multiple Users.xlsx' file.
</commit_message>
<xml_diff>
--- a/clustered_rounds.xlsx
+++ b/clustered_rounds.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,11 +596,11 @@
         <v>-9.44</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         <v>-8.380000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -746,7 +746,7 @@
         <v>-7.96</v>
       </c>
       <c r="M6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -796,11 +796,11 @@
         <v>-2.38</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -846,11 +846,11 @@
         <v>-9.539999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -896,11 +896,11 @@
         <v>-10.28</v>
       </c>
       <c r="M9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -946,11 +946,11 @@
         <v>-10.54</v>
       </c>
       <c r="M10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -996,11 +996,11 @@
         <v>-9.960000000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -1046,11 +1046,11 @@
         <v>-9.119999999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -1146,11 +1146,11 @@
         <v>-4.54</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1246,11 +1246,11 @@
         <v>-10.44</v>
       </c>
       <c r="M16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -1296,11 +1296,11 @@
         <v>-10.28</v>
       </c>
       <c r="M17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -1346,11 +1346,11 @@
         <v>-6.8</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1396,61 +1396,61 @@
         <v>-7.38</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ryan</t>
+          <t>Rich</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>45453</v>
+        <v>46173</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Willow Creek Hamlet Course</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G20" t="n">
-        <v>1.944</v>
+        <v>1.833</v>
       </c>
       <c r="H20" t="n">
         <v>0.056</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>0.214</v>
       </c>
       <c r="J20" t="n">
-        <v>-1.95</v>
+        <v>-1.2</v>
       </c>
       <c r="K20" t="n">
-        <v>-9.516999999999999</v>
+        <v>-6.256</v>
       </c>
       <c r="L20" t="n">
-        <v>-9.380000000000001</v>
+        <v>-7.38</v>
       </c>
       <c r="M20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Off Day</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1461,46 +1461,46 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>45492</v>
+        <v>45453</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Willow Creek Hamlet Course</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>1.889</v>
+        <v>1.944</v>
       </c>
       <c r="H21" t="n">
         <v>0.056</v>
       </c>
       <c r="I21" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>-0.15</v>
+        <v>-1.95</v>
       </c>
       <c r="K21" t="n">
-        <v>-8.1</v>
+        <v>-9.516999999999999</v>
       </c>
       <c r="L21" t="n">
-        <v>-8.380000000000001</v>
+        <v>-9.380000000000001</v>
       </c>
       <c r="M21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Off Day</t>
         </is>
       </c>
     </row>
@@ -1511,46 +1511,46 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>45520</v>
+        <v>45492</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Middle Island Country Club - Oak and Spruce</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
         <v>7</v>
       </c>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>1.889</v>
       </c>
       <c r="H22" t="n">
-        <v>0.222</v>
+        <v>0.056</v>
       </c>
       <c r="I22" t="n">
         <v>0.5</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>-0.15</v>
       </c>
       <c r="K22" t="n">
-        <v>-2.253</v>
+        <v>-8.1</v>
       </c>
       <c r="L22" t="n">
-        <v>-9.119999999999999</v>
+        <v>-8.380000000000001</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1561,46 +1561,46 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>45765</v>
+        <v>45520</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Cherry Creek</t>
+          <t>Middle Island Country Club - Oak and Spruce</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" t="n">
+        <v>7</v>
+      </c>
+      <c r="G23" t="n">
         <v>2</v>
       </c>
-      <c r="F23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G23" t="n">
-        <v>2.333</v>
-      </c>
       <c r="H23" t="n">
-        <v>0.111</v>
+        <v>0.222</v>
       </c>
       <c r="I23" t="n">
-        <v>0.357</v>
+        <v>0.5</v>
       </c>
       <c r="J23" t="n">
-        <v>-0.45</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>-8.739000000000001</v>
+        <v>-2.253</v>
       </c>
       <c r="L23" t="n">
-        <v>-15.96</v>
+        <v>-9.119999999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Off Day</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -1611,46 +1611,46 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>45853</v>
+        <v>45765</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pine Hollow</t>
+          <t>Cherry Creek</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G24" t="n">
-        <v>2.5</v>
+        <v>2.333</v>
       </c>
       <c r="H24" t="n">
         <v>0.111</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>0.357</v>
       </c>
       <c r="J24" t="n">
-        <v>-2.1</v>
+        <v>-0.45</v>
       </c>
       <c r="K24" t="n">
-        <v>-3.373</v>
+        <v>-8.739000000000001</v>
       </c>
       <c r="L24" t="n">
-        <v>-18.96</v>
+        <v>-15.96</v>
       </c>
       <c r="M24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Off Day</t>
         </is>
       </c>
     </row>
@@ -1661,96 +1661,96 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45894</v>
+        <v>45853</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Willow Creek Hamlet Course</t>
+          <t>Pine Hollow</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="K25" t="n">
+        <v>-3.373</v>
+      </c>
+      <c r="L25" t="n">
+        <v>-18.96</v>
+      </c>
+      <c r="M25" t="n">
         <v>3</v>
       </c>
-      <c r="F25" t="n">
-        <v>3</v>
-      </c>
-      <c r="G25" t="n">
-        <v>2.333</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0.214</v>
-      </c>
-      <c r="J25" t="n">
-        <v>-1.05</v>
-      </c>
-      <c r="K25" t="n">
-        <v>-9.436999999999999</v>
-      </c>
-      <c r="L25" t="n">
-        <v>-15.54</v>
-      </c>
-      <c r="M25" t="n">
-        <v>1</v>
-      </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Off Day</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>45048</v>
+        <v>45894</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Willow Creek Hamlet Course</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E26" t="n">
         <v>3</v>
       </c>
       <c r="F26" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G26" t="n">
-        <v>2</v>
+        <v>2.333</v>
       </c>
       <c r="H26" t="n">
         <v>0.167</v>
       </c>
       <c r="I26" t="n">
-        <v>0.643</v>
+        <v>0.214</v>
       </c>
       <c r="J26" t="n">
-        <v>0.6</v>
+        <v>-1.05</v>
       </c>
       <c r="K26" t="n">
-        <v>-4.753</v>
+        <v>-9.436999999999999</v>
       </c>
       <c r="L26" t="n">
-        <v>-9.539999999999999</v>
+        <v>-15.54</v>
       </c>
       <c r="M26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Off Day</t>
         </is>
       </c>
     </row>
@@ -1761,46 +1761,46 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45050</v>
+        <v>45048</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G27" t="n">
-        <v>2.056</v>
+        <v>2</v>
       </c>
       <c r="H27" t="n">
-        <v>0.222</v>
+        <v>0.167</v>
       </c>
       <c r="I27" t="n">
-        <v>0.5</v>
+        <v>0.643</v>
       </c>
       <c r="J27" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K27" t="n">
+        <v>-4.753</v>
+      </c>
+      <c r="L27" t="n">
+        <v>-9.539999999999999</v>
+      </c>
+      <c r="M27" t="n">
         <v>0</v>
       </c>
-      <c r="K27" t="n">
-        <v>-4.418</v>
-      </c>
-      <c r="L27" t="n">
-        <v>-10.12</v>
-      </c>
-      <c r="M27" t="n">
-        <v>2</v>
-      </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45053</v>
+        <v>45050</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1840,17 +1840,17 @@
         <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>-3.498</v>
+        <v>-4.418</v>
       </c>
       <c r="L28" t="n">
         <v>-10.12</v>
       </c>
       <c r="M28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1865,42 +1865,42 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G29" t="n">
-        <v>2</v>
+        <v>2.056</v>
       </c>
       <c r="H29" t="n">
-        <v>0.111</v>
+        <v>0.222</v>
       </c>
       <c r="I29" t="n">
-        <v>0.429</v>
+        <v>0.5</v>
       </c>
       <c r="J29" t="n">
-        <v>-0.3</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>-5.631</v>
+        <v>-3.498</v>
       </c>
       <c r="L29" t="n">
-        <v>-9.960000000000001</v>
+        <v>-10.12</v>
       </c>
       <c r="M29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1911,15 +1911,15 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45084</v>
+        <v>45053</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E30" t="n">
         <v>2</v>
@@ -1928,7 +1928,7 @@
         <v>6</v>
       </c>
       <c r="G30" t="n">
-        <v>2.056</v>
+        <v>2</v>
       </c>
       <c r="H30" t="n">
         <v>0.111</v>
@@ -1940,17 +1940,17 @@
         <v>-0.3</v>
       </c>
       <c r="K30" t="n">
-        <v>-4.333</v>
+        <v>-5.631</v>
       </c>
       <c r="L30" t="n">
-        <v>-10.96</v>
+        <v>-9.960000000000001</v>
       </c>
       <c r="M30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45114</v>
+        <v>45084</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1969,38 +1969,38 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E31" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G31" t="n">
-        <v>1.778</v>
+        <v>2.056</v>
       </c>
       <c r="H31" t="n">
-        <v>0.278</v>
+        <v>0.111</v>
       </c>
       <c r="I31" t="n">
-        <v>0.214</v>
+        <v>0.429</v>
       </c>
       <c r="J31" t="n">
-        <v>-1.05</v>
+        <v>-0.3</v>
       </c>
       <c r="K31" t="n">
-        <v>-6.473</v>
+        <v>-4.333</v>
       </c>
       <c r="L31" t="n">
-        <v>-5.1</v>
+        <v>-10.96</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45136</v>
+        <v>45114</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -2019,31 +2019,31 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" t="n">
         <v>3</v>
       </c>
-      <c r="F32" t="n">
-        <v>6</v>
-      </c>
       <c r="G32" t="n">
-        <v>1.722</v>
+        <v>1.778</v>
       </c>
       <c r="H32" t="n">
-        <v>0.167</v>
+        <v>0.278</v>
       </c>
       <c r="I32" t="n">
-        <v>0.429</v>
+        <v>0.214</v>
       </c>
       <c r="J32" t="n">
-        <v>-0.15</v>
+        <v>-1.05</v>
       </c>
       <c r="K32" t="n">
-        <v>-0.2</v>
+        <v>-6.473</v>
       </c>
       <c r="L32" t="n">
-        <v>-0.6</v>
+        <v>-5.1</v>
       </c>
       <c r="M32" t="n">
         <v>4</v>
@@ -2061,46 +2061,46 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45137</v>
+        <v>45136</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G33" t="n">
-        <v>1.778</v>
+        <v>1.722</v>
       </c>
       <c r="H33" t="n">
-        <v>0.222</v>
+        <v>0.167</v>
       </c>
       <c r="I33" t="n">
-        <v>0.286</v>
+        <v>0.429</v>
       </c>
       <c r="J33" t="n">
-        <v>-0.9</v>
+        <v>-0.15</v>
       </c>
       <c r="K33" t="n">
-        <v>-4.631</v>
+        <v>-0.2</v>
       </c>
       <c r="L33" t="n">
-        <v>-5.12</v>
+        <v>-0.6</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45143</v>
+        <v>45137</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -2119,38 +2119,38 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="E34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G34" t="n">
-        <v>2.167</v>
+        <v>1.778</v>
       </c>
       <c r="H34" t="n">
-        <v>0.278</v>
+        <v>0.222</v>
       </c>
       <c r="I34" t="n">
-        <v>0.429</v>
+        <v>0.286</v>
       </c>
       <c r="J34" t="n">
-        <v>-0.3</v>
+        <v>-0.9</v>
       </c>
       <c r="K34" t="n">
-        <v>-2.051</v>
+        <v>-4.631</v>
       </c>
       <c r="L34" t="n">
-        <v>-11.7</v>
+        <v>-5.12</v>
       </c>
       <c r="M34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2161,46 +2161,46 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45144</v>
+        <v>45143</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Bethpage Black</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E35" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" t="n">
+        <v>6</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2.167</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="J35" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="K35" t="n">
+        <v>-2.051</v>
+      </c>
+      <c r="L35" t="n">
+        <v>-11.7</v>
+      </c>
+      <c r="M35" t="n">
         <v>1</v>
       </c>
-      <c r="F35" t="n">
-        <v>8</v>
-      </c>
-      <c r="G35" t="n">
-        <v>1.778</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0.056</v>
-      </c>
-      <c r="I35" t="n">
-        <v>0.571</v>
-      </c>
-      <c r="J35" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="K35" t="n">
-        <v>-3.02</v>
-      </c>
-      <c r="L35" t="n">
-        <v>-6.38</v>
-      </c>
-      <c r="M35" t="n">
-        <v>3</v>
-      </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2211,46 +2211,46 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45156</v>
+        <v>45144</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Middle Island Country Club - Oak and Spruce</t>
+          <t>Bethpage Black</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G36" t="n">
-        <v>1.944</v>
+        <v>1.778</v>
       </c>
       <c r="H36" t="n">
-        <v>0.222</v>
+        <v>0.056</v>
       </c>
       <c r="I36" t="n">
-        <v>0.429</v>
+        <v>0.571</v>
       </c>
       <c r="J36" t="n">
-        <v>-0.3</v>
+        <v>0.3</v>
       </c>
       <c r="K36" t="n">
-        <v>-2.253</v>
+        <v>-3.02</v>
       </c>
       <c r="L36" t="n">
-        <v>-8.119999999999999</v>
+        <v>-6.38</v>
       </c>
       <c r="M36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2261,46 +2261,46 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45172</v>
+        <v>45156</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Middle Island Country Club - Oak and Spruce</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E37" t="n">
+        <v>4</v>
+      </c>
+      <c r="F37" t="n">
         <v>6</v>
       </c>
-      <c r="F37" t="n">
-        <v>8</v>
-      </c>
       <c r="G37" t="n">
-        <v>2.056</v>
+        <v>1.944</v>
       </c>
       <c r="H37" t="n">
-        <v>0.333</v>
+        <v>0.222</v>
       </c>
       <c r="I37" t="n">
-        <v>0.571</v>
+        <v>0.429</v>
       </c>
       <c r="J37" t="n">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="K37" t="n">
-        <v>-1.498</v>
+        <v>-2.253</v>
       </c>
       <c r="L37" t="n">
-        <v>-9.279999999999999</v>
+        <v>-8.119999999999999</v>
       </c>
       <c r="M37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2311,46 +2311,46 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45434</v>
+        <v>45172</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E38" t="n">
         <v>6</v>
       </c>
       <c r="F38" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G38" t="n">
-        <v>2.111</v>
+        <v>2.056</v>
       </c>
       <c r="H38" t="n">
         <v>0.333</v>
       </c>
       <c r="I38" t="n">
-        <v>0.214</v>
+        <v>0.571</v>
       </c>
       <c r="J38" t="n">
-        <v>-1.2</v>
+        <v>0.3</v>
       </c>
       <c r="K38" t="n">
-        <v>-2.471</v>
+        <v>-1.498</v>
       </c>
       <c r="L38" t="n">
-        <v>-10.28</v>
+        <v>-9.279999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45440</v>
+        <v>45434</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -2369,38 +2369,38 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F39" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G39" t="n">
-        <v>1.833</v>
+        <v>2.111</v>
       </c>
       <c r="H39" t="n">
-        <v>0.111</v>
+        <v>0.333</v>
       </c>
       <c r="I39" t="n">
-        <v>0.571</v>
+        <v>0.214</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="K39" t="n">
-        <v>-5.711</v>
+        <v>-2.471</v>
       </c>
       <c r="L39" t="n">
-        <v>-6.96</v>
+        <v>-10.28</v>
       </c>
       <c r="M39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2411,39 +2411,39 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45443</v>
+        <v>45440</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E40" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G40" t="n">
-        <v>1.944</v>
+        <v>1.833</v>
       </c>
       <c r="H40" t="n">
-        <v>0.333</v>
+        <v>0.111</v>
       </c>
       <c r="I40" t="n">
-        <v>0.286</v>
+        <v>0.571</v>
       </c>
       <c r="J40" t="n">
-        <v>-0.9</v>
+        <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>-1.498</v>
+        <v>-5.711</v>
       </c>
       <c r="L40" t="n">
-        <v>-7.28</v>
+        <v>-6.96</v>
       </c>
       <c r="M40" t="n">
         <v>0</v>
@@ -2461,46 +2461,46 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45453</v>
+        <v>45443</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Willow Creek Hamlet Course</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D41" t="n">
         <v>35</v>
       </c>
       <c r="E41" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G41" t="n">
         <v>1.944</v>
       </c>
       <c r="H41" t="n">
-        <v>0.167</v>
+        <v>0.333</v>
       </c>
       <c r="I41" t="n">
-        <v>0.357</v>
+        <v>0.286</v>
       </c>
       <c r="J41" t="n">
-        <v>-0.45</v>
+        <v>-0.9</v>
       </c>
       <c r="K41" t="n">
-        <v>-5.437</v>
+        <v>-1.498</v>
       </c>
       <c r="L41" t="n">
-        <v>-8.539999999999999</v>
+        <v>-7.28</v>
       </c>
       <c r="M41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2511,46 +2511,46 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45465</v>
+        <v>45453</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Wind Watch Hamlet Course</t>
+          <t>Willow Creek Hamlet Course</t>
         </is>
       </c>
       <c r="D42" t="n">
         <v>35</v>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G42" t="n">
         <v>1.944</v>
       </c>
       <c r="H42" t="n">
-        <v>0.111</v>
+        <v>0.167</v>
       </c>
       <c r="I42" t="n">
-        <v>0.214</v>
+        <v>0.357</v>
       </c>
       <c r="J42" t="n">
-        <v>-1.2</v>
+        <v>-0.45</v>
       </c>
       <c r="K42" t="n">
-        <v>-5.476</v>
+        <v>-5.437</v>
       </c>
       <c r="L42" t="n">
-        <v>-8.960000000000001</v>
+        <v>-8.539999999999999</v>
       </c>
       <c r="M42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2561,39 +2561,39 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45466</v>
+        <v>45465</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Bethpage Red</t>
+          <t>Wind Watch Hamlet Course</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E43" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F43" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G43" t="n">
-        <v>1.667</v>
+        <v>1.944</v>
       </c>
       <c r="H43" t="n">
-        <v>0.222</v>
+        <v>0.111</v>
       </c>
       <c r="I43" t="n">
-        <v>0.5</v>
+        <v>0.214</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="K43" t="n">
-        <v>-1.818</v>
+        <v>-5.476</v>
       </c>
       <c r="L43" t="n">
-        <v>-3.12</v>
+        <v>-8.960000000000001</v>
       </c>
       <c r="M43" t="n">
         <v>4</v>
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45467</v>
+        <v>45466</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Bethpage Red</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E44" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F44" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G44" t="n">
-        <v>1.833</v>
+        <v>1.667</v>
       </c>
       <c r="H44" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="I44" t="n">
         <v>0.5</v>
       </c>
-      <c r="I44" t="n">
-        <v>0.429</v>
-      </c>
       <c r="J44" t="n">
-        <v>-0.3</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>-0.976</v>
+        <v>-1.818</v>
       </c>
       <c r="L44" t="n">
-        <v>-4.02</v>
+        <v>-3.12</v>
       </c>
       <c r="M44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45475</v>
+        <v>45467</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -2669,38 +2669,38 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E45" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F45" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G45" t="n">
-        <v>1.611</v>
+        <v>1.833</v>
       </c>
       <c r="H45" t="n">
-        <v>0.444</v>
+        <v>0.5</v>
       </c>
       <c r="I45" t="n">
-        <v>0.571</v>
+        <v>0.429</v>
       </c>
       <c r="J45" t="n">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="K45" t="n">
-        <v>-0.253</v>
+        <v>-0.976</v>
       </c>
       <c r="L45" t="n">
-        <v>-0.44</v>
+        <v>-4.02</v>
       </c>
       <c r="M45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -2711,27 +2711,27 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45480</v>
+        <v>45475</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Bethpage Red</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F46" t="n">
         <v>8</v>
       </c>
       <c r="G46" t="n">
-        <v>1.667</v>
+        <v>1.611</v>
       </c>
       <c r="H46" t="n">
-        <v>0.111</v>
+        <v>0.444</v>
       </c>
       <c r="I46" t="n">
         <v>0.571</v>
@@ -2740,10 +2740,10 @@
         <v>0.3</v>
       </c>
       <c r="K46" t="n">
-        <v>-2.422</v>
+        <v>-0.253</v>
       </c>
       <c r="L46" t="n">
-        <v>-3.96</v>
+        <v>-0.44</v>
       </c>
       <c r="M46" t="n">
         <v>3</v>
@@ -2761,46 +2761,46 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45487</v>
+        <v>45480</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Red</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E47" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G47" t="n">
-        <v>1.611</v>
+        <v>1.667</v>
       </c>
       <c r="H47" t="n">
-        <v>0.333</v>
+        <v>0.111</v>
       </c>
       <c r="I47" t="n">
-        <v>0.214</v>
+        <v>0.571</v>
       </c>
       <c r="J47" t="n">
-        <v>-1.2</v>
+        <v>0.3</v>
       </c>
       <c r="K47" t="n">
-        <v>-1.578</v>
+        <v>-2.422</v>
       </c>
       <c r="L47" t="n">
-        <v>-1.28</v>
+        <v>-3.96</v>
       </c>
       <c r="M47" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2811,46 +2811,46 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45492</v>
+        <v>45487</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D48" t="n">
         <v>29</v>
       </c>
       <c r="E48" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F48" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G48" t="n">
         <v>1.611</v>
       </c>
       <c r="H48" t="n">
-        <v>0.278</v>
+        <v>0.333</v>
       </c>
       <c r="I48" t="n">
-        <v>0.571</v>
+        <v>0.214</v>
       </c>
       <c r="J48" t="n">
-        <v>0.15</v>
+        <v>-1.2</v>
       </c>
       <c r="K48" t="n">
-        <v>-3.1</v>
+        <v>-1.578</v>
       </c>
       <c r="L48" t="n">
-        <v>-1.7</v>
+        <v>-1.28</v>
       </c>
       <c r="M48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45496</v>
+        <v>45492</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -2869,38 +2869,38 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G49" t="n">
-        <v>1.5</v>
+        <v>1.611</v>
       </c>
       <c r="H49" t="n">
-        <v>0.167</v>
+        <v>0.278</v>
       </c>
       <c r="I49" t="n">
-        <v>0.643</v>
+        <v>0.571</v>
       </c>
       <c r="J49" t="n">
-        <v>0.45</v>
+        <v>0.15</v>
       </c>
       <c r="K49" t="n">
-        <v>-4.1</v>
+        <v>-3.1</v>
       </c>
       <c r="L49" t="n">
-        <v>-0.54</v>
+        <v>-1.7</v>
       </c>
       <c r="M49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2911,46 +2911,46 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>45502</v>
+        <v>45496</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F50" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G50" t="n">
-        <v>1.611</v>
+        <v>1.5</v>
       </c>
       <c r="H50" t="n">
-        <v>0.222</v>
+        <v>0.167</v>
       </c>
       <c r="I50" t="n">
-        <v>0.429</v>
+        <v>0.643</v>
       </c>
       <c r="J50" t="n">
-        <v>-0.3</v>
+        <v>0.45</v>
       </c>
       <c r="K50" t="n">
-        <v>-3.578</v>
+        <v>-4.1</v>
       </c>
       <c r="L50" t="n">
-        <v>-2.12</v>
+        <v>-0.54</v>
       </c>
       <c r="M50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2961,15 +2961,15 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>45514</v>
+        <v>45502</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E51" t="n">
         <v>4</v>
@@ -2978,7 +2978,7 @@
         <v>6</v>
       </c>
       <c r="G51" t="n">
-        <v>1.722</v>
+        <v>1.611</v>
       </c>
       <c r="H51" t="n">
         <v>0.222</v>
@@ -2987,20 +2987,20 @@
         <v>0.429</v>
       </c>
       <c r="J51" t="n">
-        <v>-0.45</v>
+        <v>-0.3</v>
       </c>
       <c r="K51" t="n">
-        <v>-3.6</v>
+        <v>-3.578</v>
       </c>
       <c r="L51" t="n">
-        <v>-4.12</v>
+        <v>-2.12</v>
       </c>
       <c r="M51" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3011,46 +3011,46 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>45535</v>
+        <v>45514</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F52" t="n">
         <v>6</v>
       </c>
       <c r="G52" t="n">
-        <v>1.778</v>
+        <v>1.722</v>
       </c>
       <c r="H52" t="n">
-        <v>0.167</v>
+        <v>0.222</v>
       </c>
       <c r="I52" t="n">
         <v>0.429</v>
       </c>
       <c r="J52" t="n">
-        <v>-0.3</v>
+        <v>-0.45</v>
       </c>
       <c r="K52" t="n">
-        <v>-5.433</v>
+        <v>-3.6</v>
       </c>
       <c r="L52" t="n">
-        <v>-5.54</v>
+        <v>-4.12</v>
       </c>
       <c r="M52" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3061,39 +3061,39 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>45570</v>
+        <v>45535</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E53" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F53" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G53" t="n">
-        <v>1.611</v>
+        <v>1.778</v>
       </c>
       <c r="H53" t="n">
-        <v>0.278</v>
+        <v>0.167</v>
       </c>
       <c r="I53" t="n">
-        <v>0.357</v>
+        <v>0.429</v>
       </c>
       <c r="J53" t="n">
-        <v>-0.6</v>
+        <v>-0.3</v>
       </c>
       <c r="K53" t="n">
-        <v>-3.676</v>
+        <v>-5.433</v>
       </c>
       <c r="L53" t="n">
-        <v>-2.12</v>
+        <v>-5.54</v>
       </c>
       <c r="M53" t="n">
         <v>4</v>
@@ -3111,11 +3111,11 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>45580</v>
+        <v>45570</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Sebonack Golf Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3125,7 +3125,7 @@
         <v>5</v>
       </c>
       <c r="F54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G54" t="n">
         <v>1.611</v>
@@ -3134,23 +3134,23 @@
         <v>0.278</v>
       </c>
       <c r="I54" t="n">
-        <v>0.429</v>
+        <v>0.357</v>
       </c>
       <c r="J54" t="n">
-        <v>-0.3</v>
+        <v>-0.6</v>
       </c>
       <c r="K54" t="n">
-        <v>-3.789</v>
+        <v>-3.676</v>
       </c>
       <c r="L54" t="n">
-        <v>-1.7</v>
+        <v>-2.12</v>
       </c>
       <c r="M54" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3161,39 +3161,39 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45649</v>
+        <v>45580</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Ka'anapali Golf Resort Royal Course</t>
+          <t>Sebonack Golf Club</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F55" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G55" t="n">
-        <v>1.944</v>
+        <v>1.611</v>
       </c>
       <c r="H55" t="n">
-        <v>0.056</v>
+        <v>0.278</v>
       </c>
       <c r="I55" t="n">
-        <v>0.357</v>
+        <v>0.429</v>
       </c>
       <c r="J55" t="n">
-        <v>-0.6</v>
+        <v>-0.3</v>
       </c>
       <c r="K55" t="n">
-        <v>-4.167</v>
+        <v>-3.789</v>
       </c>
       <c r="L55" t="n">
-        <v>-9.380000000000001</v>
+        <v>-1.7</v>
       </c>
       <c r="M55" t="n">
         <v>2</v>
@@ -3211,42 +3211,42 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>45653</v>
+        <v>45649</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Wailea Golf Club Gold Course</t>
+          <t>Ka'anapali Golf Resort Royal Course</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="n">
         <v>5</v>
       </c>
-      <c r="F56" t="n">
-        <v>3</v>
-      </c>
       <c r="G56" t="n">
-        <v>1.722</v>
+        <v>1.944</v>
       </c>
       <c r="H56" t="n">
-        <v>0.278</v>
+        <v>0.056</v>
       </c>
       <c r="I56" t="n">
-        <v>0.214</v>
+        <v>0.357</v>
       </c>
       <c r="J56" t="n">
-        <v>0.3</v>
+        <v>-0.6</v>
       </c>
       <c r="K56" t="n">
-        <v>-1.651</v>
+        <v>-4.167</v>
       </c>
       <c r="L56" t="n">
-        <v>-3.7</v>
+        <v>-9.380000000000001</v>
       </c>
       <c r="M56" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
@@ -3261,46 +3261,46 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>45655</v>
+        <v>45653</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Wailea Golf Club Emerald Course</t>
+          <t>Wailea Golf Club Gold Course</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F57" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="G57" t="n">
-        <v>1.889</v>
+        <v>1.722</v>
       </c>
       <c r="H57" t="n">
-        <v>0.333</v>
+        <v>0.278</v>
       </c>
       <c r="I57" t="n">
-        <v>0.786</v>
+        <v>0.214</v>
       </c>
       <c r="J57" t="n">
-        <v>1.2</v>
+        <v>0.3</v>
       </c>
       <c r="K57" t="n">
-        <v>-1.556</v>
+        <v>-1.651</v>
       </c>
       <c r="L57" t="n">
-        <v>-6.28</v>
+        <v>-3.7</v>
       </c>
       <c r="M57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3311,46 +3311,46 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>45735</v>
+        <v>45655</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Wailea Golf Club Emerald Course</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E58" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F58" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G58" t="n">
-        <v>1.722</v>
+        <v>1.889</v>
       </c>
       <c r="H58" t="n">
-        <v>0.556</v>
+        <v>0.333</v>
       </c>
       <c r="I58" t="n">
-        <v>0.5</v>
+        <v>0.786</v>
       </c>
       <c r="J58" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K58" t="n">
+        <v>-1.556</v>
+      </c>
+      <c r="L58" t="n">
+        <v>-6.28</v>
+      </c>
+      <c r="M58" t="n">
         <v>0</v>
       </c>
-      <c r="K58" t="n">
-        <v>-0.676</v>
-      </c>
-      <c r="L58" t="n">
-        <v>-1.6</v>
-      </c>
-      <c r="M58" t="n">
-        <v>1</v>
-      </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -3361,46 +3361,46 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>45829</v>
+        <v>45735</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E59" t="n">
+        <v>10</v>
+      </c>
+      <c r="F59" t="n">
         <v>7</v>
       </c>
-      <c r="F59" t="n">
-        <v>9</v>
-      </c>
       <c r="G59" t="n">
-        <v>1.556</v>
+        <v>1.722</v>
       </c>
       <c r="H59" t="n">
-        <v>0.389</v>
+        <v>0.556</v>
       </c>
       <c r="I59" t="n">
-        <v>0.643</v>
+        <v>0.5</v>
       </c>
       <c r="J59" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="K59" t="n">
-        <v>-1.45</v>
+        <v>-0.676</v>
       </c>
       <c r="L59" t="n">
-        <v>0.14</v>
+        <v>-1.6</v>
       </c>
       <c r="M59" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -3411,46 +3411,46 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>45831</v>
+        <v>45829</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E60" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F60" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G60" t="n">
-        <v>1.778</v>
+        <v>1.556</v>
       </c>
       <c r="H60" t="n">
-        <v>0.444</v>
+        <v>0.389</v>
       </c>
       <c r="I60" t="n">
-        <v>0.571</v>
+        <v>0.643</v>
       </c>
       <c r="J60" t="n">
-        <v>0.3</v>
+        <v>0.45</v>
       </c>
       <c r="K60" t="n">
-        <v>0.247</v>
+        <v>-1.45</v>
       </c>
       <c r="L60" t="n">
-        <v>-3.02</v>
+        <v>0.14</v>
       </c>
       <c r="M60" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -3461,11 +3461,11 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45844</v>
+        <v>45831</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3475,7 +3475,7 @@
         <v>8</v>
       </c>
       <c r="F61" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G61" t="n">
         <v>1.778</v>
@@ -3484,23 +3484,23 @@
         <v>0.444</v>
       </c>
       <c r="I61" t="n">
-        <v>0.5</v>
+        <v>0.571</v>
       </c>
       <c r="J61" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="K61" t="n">
-        <v>-1.596</v>
+        <v>0.247</v>
       </c>
       <c r="L61" t="n">
-        <v>-3.44</v>
+        <v>-3.02</v>
       </c>
       <c r="M61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45857</v>
+        <v>45844</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -3519,38 +3519,38 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E62" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F62" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G62" t="n">
-        <v>1.833</v>
+        <v>1.778</v>
       </c>
       <c r="H62" t="n">
-        <v>0.611</v>
+        <v>0.444</v>
       </c>
       <c r="I62" t="n">
-        <v>0.571</v>
+        <v>0.5</v>
       </c>
       <c r="J62" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>0.904</v>
+        <v>-1.596</v>
       </c>
       <c r="L62" t="n">
-        <v>-3.18</v>
+        <v>-3.44</v>
       </c>
       <c r="M62" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -3561,46 +3561,46 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>45868</v>
+        <v>45857</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Bethpage Red</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E63" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F63" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G63" t="n">
-        <v>1.611</v>
+        <v>1.833</v>
       </c>
       <c r="H63" t="n">
-        <v>0.222</v>
+        <v>0.611</v>
       </c>
       <c r="I63" t="n">
-        <v>0.5</v>
+        <v>0.571</v>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K63" t="n">
-        <v>-1.342</v>
+        <v>0.904</v>
       </c>
       <c r="L63" t="n">
-        <v>-2.12</v>
+        <v>-3.18</v>
       </c>
       <c r="M63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -3611,46 +3611,46 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45886</v>
+        <v>45868</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Spring Lake Thunderbird</t>
+          <t>Bethpage Red</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E64" t="n">
         <v>4</v>
       </c>
       <c r="F64" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G64" t="n">
-        <v>1.667</v>
+        <v>1.611</v>
       </c>
       <c r="H64" t="n">
         <v>0.222</v>
       </c>
       <c r="I64" t="n">
-        <v>0.786</v>
+        <v>0.5</v>
       </c>
       <c r="J64" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="K64" t="n">
-        <v>-3.573</v>
+        <v>-1.342</v>
       </c>
       <c r="L64" t="n">
-        <v>-3.12</v>
+        <v>-2.12</v>
       </c>
       <c r="M64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>45892</v>
+        <v>45886</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -3669,38 +3669,38 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E65" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F65" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G65" t="n">
-        <v>1.778</v>
+        <v>1.667</v>
       </c>
       <c r="H65" t="n">
-        <v>0.278</v>
+        <v>0.222</v>
       </c>
       <c r="I65" t="n">
-        <v>0.429</v>
+        <v>0.786</v>
       </c>
       <c r="J65" t="n">
-        <v>-0.3</v>
+        <v>1.2</v>
       </c>
       <c r="K65" t="n">
-        <v>-3.153</v>
+        <v>-3.573</v>
       </c>
       <c r="L65" t="n">
-        <v>-4.7</v>
+        <v>-3.12</v>
       </c>
       <c r="M65" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -3711,39 +3711,39 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>45894</v>
+        <v>45892</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Willow Creek Hamlet Course</t>
+          <t>Spring Lake Thunderbird</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E66" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F66" t="n">
         <v>6</v>
       </c>
       <c r="G66" t="n">
-        <v>2.111</v>
+        <v>1.778</v>
       </c>
       <c r="H66" t="n">
-        <v>0.056</v>
+        <v>0.278</v>
       </c>
       <c r="I66" t="n">
         <v>0.429</v>
       </c>
       <c r="J66" t="n">
-        <v>-0.15</v>
+        <v>-0.3</v>
       </c>
       <c r="K66" t="n">
-        <v>-5.517</v>
+        <v>-3.153</v>
       </c>
       <c r="L66" t="n">
-        <v>-12.38</v>
+        <v>-4.7</v>
       </c>
       <c r="M66" t="n">
         <v>2</v>
@@ -3761,46 +3761,46 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>45897</v>
+        <v>45894</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Spring Lake Thunderbird</t>
+          <t>Willow Creek Hamlet Course</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E67" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F67" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G67" t="n">
-        <v>1.722</v>
+        <v>2.111</v>
       </c>
       <c r="H67" t="n">
-        <v>0.222</v>
+        <v>0.056</v>
       </c>
       <c r="I67" t="n">
-        <v>0.214</v>
+        <v>0.429</v>
       </c>
       <c r="J67" t="n">
-        <v>-1.2</v>
+        <v>-0.15</v>
       </c>
       <c r="K67" t="n">
-        <v>-5.733</v>
+        <v>-5.517</v>
       </c>
       <c r="L67" t="n">
-        <v>-4.12</v>
+        <v>-12.38</v>
       </c>
       <c r="M67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3811,27 +3811,27 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>45941</v>
+        <v>45897</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Wind Watch Hamlet Course</t>
+          <t>Spring Lake Thunderbird</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E68" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F68" t="n">
         <v>3</v>
       </c>
       <c r="G68" t="n">
-        <v>1.667</v>
+        <v>1.722</v>
       </c>
       <c r="H68" t="n">
-        <v>0.056</v>
+        <v>0.222</v>
       </c>
       <c r="I68" t="n">
         <v>0.214</v>
@@ -3840,17 +3840,17 @@
         <v>-1.2</v>
       </c>
       <c r="K68" t="n">
-        <v>-5.522</v>
+        <v>-5.733</v>
       </c>
       <c r="L68" t="n">
-        <v>-4.38</v>
+        <v>-4.12</v>
       </c>
       <c r="M68" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3861,42 +3861,42 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>46160</v>
+        <v>45941</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Wind Watch Hamlet Course</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E69" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F69" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G69" t="n">
-        <v>1.889</v>
+        <v>1.667</v>
       </c>
       <c r="H69" t="n">
-        <v>0.444</v>
+        <v>0.056</v>
       </c>
       <c r="I69" t="n">
-        <v>0.357</v>
+        <v>0.214</v>
       </c>
       <c r="J69" t="n">
-        <v>-0.6</v>
+        <v>-1.2</v>
       </c>
       <c r="K69" t="n">
-        <v>-0.173</v>
+        <v>-5.522</v>
       </c>
       <c r="L69" t="n">
-        <v>-5.44</v>
+        <v>-4.38</v>
       </c>
       <c r="M69" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -3911,39 +3911,39 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>46164</v>
+        <v>46160</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F70" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G70" t="n">
-        <v>1.722</v>
+        <v>1.889</v>
       </c>
       <c r="H70" t="n">
-        <v>0.111</v>
+        <v>0.444</v>
       </c>
       <c r="I70" t="n">
-        <v>0.643</v>
+        <v>0.357</v>
       </c>
       <c r="J70" t="n">
-        <v>0.45</v>
+        <v>-0.6</v>
       </c>
       <c r="K70" t="n">
-        <v>-3.95</v>
+        <v>-0.173</v>
       </c>
       <c r="L70" t="n">
-        <v>-4.96</v>
+        <v>-5.44</v>
       </c>
       <c r="M70" t="n">
         <v>3</v>
@@ -3951,6 +3951,106 @@
       <c r="N70" t="inlineStr">
         <is>
           <t>Fairway Putter</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>46164</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Brentwood Country Club</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>31</v>
+      </c>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="n">
+        <v>9</v>
+      </c>
+      <c r="G71" t="n">
+        <v>1.722</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K71" t="n">
+        <v>-3.95</v>
+      </c>
+      <c r="L71" t="n">
+        <v>-4.96</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>All Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Bethpage Green</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>35</v>
+      </c>
+      <c r="E72" t="n">
+        <v>5</v>
+      </c>
+      <c r="F72" t="n">
+        <v>5</v>
+      </c>
+      <c r="G72" t="n">
+        <v>1.944</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0.357</v>
+      </c>
+      <c r="J72" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="K72" t="n">
+        <v>-3.256</v>
+      </c>
+      <c r="L72" t="n">
+        <v>-7.7</v>
+      </c>
+      <c r="M72" t="n">
+        <v>1</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update multiple Excel files and Golf Analytics notebook to standardize execution counts to null for improved consistency in analysis. Changes include club ranges, club selector, clustered rounds, clutch score analysis, golf recommendations, strokes gained summary, and Golf Dashboard 2.0.
</commit_message>
<xml_diff>
--- a/clustered_rounds.xlsx
+++ b/clustered_rounds.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1496,11 +1496,11 @@
         <v>-9.380000000000001</v>
       </c>
       <c r="M21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Off Day</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -1546,11 +1546,11 @@
         <v>-8.380000000000001</v>
       </c>
       <c r="M22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -1596,11 +1596,11 @@
         <v>-9.119999999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1696,11 +1696,11 @@
         <v>-18.96</v>
       </c>
       <c r="M25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Off Day</t>
         </is>
       </c>
     </row>
@@ -1757,50 +1757,50 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45048</v>
+        <v>46185</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Swan Lake</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>2.278</v>
       </c>
       <c r="H27" t="n">
-        <v>0.167</v>
+        <v>0.222</v>
       </c>
       <c r="I27" t="n">
-        <v>0.643</v>
+        <v>0.286</v>
       </c>
       <c r="J27" t="n">
-        <v>0.6</v>
+        <v>-0.9</v>
       </c>
       <c r="K27" t="n">
-        <v>-4.753</v>
+        <v>-2.529</v>
       </c>
       <c r="L27" t="n">
-        <v>-9.539999999999999</v>
+        <v>-14.12</v>
       </c>
       <c r="M27" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1811,46 +1811,46 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45050</v>
+        <v>45048</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G28" t="n">
-        <v>2.056</v>
+        <v>2</v>
       </c>
       <c r="H28" t="n">
-        <v>0.222</v>
+        <v>0.167</v>
       </c>
       <c r="I28" t="n">
-        <v>0.5</v>
+        <v>0.643</v>
       </c>
       <c r="J28" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K28" t="n">
+        <v>-4.753</v>
+      </c>
+      <c r="L28" t="n">
+        <v>-9.539999999999999</v>
+      </c>
+      <c r="M28" t="n">
         <v>0</v>
       </c>
-      <c r="K28" t="n">
-        <v>-4.418</v>
-      </c>
-      <c r="L28" t="n">
-        <v>-10.12</v>
-      </c>
-      <c r="M28" t="n">
-        <v>1</v>
-      </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45053</v>
+        <v>45050</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1890,7 +1890,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>-3.498</v>
+        <v>-4.418</v>
       </c>
       <c r="L29" t="n">
         <v>-10.12</v>
@@ -1915,35 +1915,35 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>2.056</v>
       </c>
       <c r="H30" t="n">
-        <v>0.111</v>
+        <v>0.222</v>
       </c>
       <c r="I30" t="n">
-        <v>0.429</v>
+        <v>0.5</v>
       </c>
       <c r="J30" t="n">
-        <v>-0.3</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>-5.631</v>
+        <v>-3.498</v>
       </c>
       <c r="L30" t="n">
-        <v>-9.960000000000001</v>
+        <v>-10.12</v>
       </c>
       <c r="M30" t="n">
         <v>1</v>
@@ -1961,15 +1961,15 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45084</v>
+        <v>45053</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E31" t="n">
         <v>2</v>
@@ -1978,7 +1978,7 @@
         <v>6</v>
       </c>
       <c r="G31" t="n">
-        <v>2.056</v>
+        <v>2</v>
       </c>
       <c r="H31" t="n">
         <v>0.111</v>
@@ -1990,10 +1990,10 @@
         <v>-0.3</v>
       </c>
       <c r="K31" t="n">
-        <v>-4.333</v>
+        <v>-5.631</v>
       </c>
       <c r="L31" t="n">
-        <v>-10.96</v>
+        <v>-9.960000000000001</v>
       </c>
       <c r="M31" t="n">
         <v>1</v>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45114</v>
+        <v>45084</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -2019,34 +2019,34 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G32" t="n">
-        <v>1.778</v>
+        <v>2.056</v>
       </c>
       <c r="H32" t="n">
-        <v>0.278</v>
+        <v>0.111</v>
       </c>
       <c r="I32" t="n">
-        <v>0.214</v>
+        <v>0.429</v>
       </c>
       <c r="J32" t="n">
-        <v>-1.05</v>
+        <v>-0.3</v>
       </c>
       <c r="K32" t="n">
-        <v>-6.473</v>
+        <v>-4.333</v>
       </c>
       <c r="L32" t="n">
-        <v>-5.1</v>
+        <v>-10.96</v>
       </c>
       <c r="M32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45136</v>
+        <v>45114</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -2069,38 +2069,38 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E33" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" t="n">
         <v>3</v>
       </c>
-      <c r="F33" t="n">
-        <v>6</v>
-      </c>
       <c r="G33" t="n">
-        <v>1.722</v>
+        <v>1.778</v>
       </c>
       <c r="H33" t="n">
-        <v>0.167</v>
+        <v>0.278</v>
       </c>
       <c r="I33" t="n">
-        <v>0.429</v>
+        <v>0.214</v>
       </c>
       <c r="J33" t="n">
-        <v>-0.15</v>
+        <v>-1.05</v>
       </c>
       <c r="K33" t="n">
-        <v>-0.2</v>
+        <v>-6.473</v>
       </c>
       <c r="L33" t="n">
-        <v>-0.6</v>
+        <v>-5.1</v>
       </c>
       <c r="M33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2111,46 +2111,46 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45137</v>
+        <v>45136</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G34" t="n">
-        <v>1.778</v>
+        <v>1.722</v>
       </c>
       <c r="H34" t="n">
-        <v>0.222</v>
+        <v>0.167</v>
       </c>
       <c r="I34" t="n">
-        <v>0.286</v>
+        <v>0.429</v>
       </c>
       <c r="J34" t="n">
-        <v>-0.9</v>
+        <v>-0.15</v>
       </c>
       <c r="K34" t="n">
-        <v>-4.631</v>
+        <v>-0.2</v>
       </c>
       <c r="L34" t="n">
-        <v>-5.12</v>
+        <v>-0.6</v>
       </c>
       <c r="M34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45143</v>
+        <v>45137</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -2169,34 +2169,34 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="E35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F35" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G35" t="n">
-        <v>2.167</v>
+        <v>1.778</v>
       </c>
       <c r="H35" t="n">
-        <v>0.278</v>
+        <v>0.222</v>
       </c>
       <c r="I35" t="n">
-        <v>0.429</v>
+        <v>0.286</v>
       </c>
       <c r="J35" t="n">
-        <v>-0.3</v>
+        <v>-0.9</v>
       </c>
       <c r="K35" t="n">
-        <v>-2.051</v>
+        <v>-4.631</v>
       </c>
       <c r="L35" t="n">
-        <v>-11.7</v>
+        <v>-5.12</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -2211,46 +2211,46 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45144</v>
+        <v>45143</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Bethpage Black</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E36" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" t="n">
+        <v>6</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2.167</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="J36" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="K36" t="n">
+        <v>-2.051</v>
+      </c>
+      <c r="L36" t="n">
+        <v>-11.7</v>
+      </c>
+      <c r="M36" t="n">
         <v>1</v>
       </c>
-      <c r="F36" t="n">
-        <v>8</v>
-      </c>
-      <c r="G36" t="n">
-        <v>1.778</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0.056</v>
-      </c>
-      <c r="I36" t="n">
-        <v>0.571</v>
-      </c>
-      <c r="J36" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="K36" t="n">
-        <v>-3.02</v>
-      </c>
-      <c r="L36" t="n">
-        <v>-6.38</v>
-      </c>
-      <c r="M36" t="n">
-        <v>0</v>
-      </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2261,46 +2261,46 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45156</v>
+        <v>45144</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Middle Island Country Club - Oak and Spruce</t>
+          <t>Bethpage Black</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G37" t="n">
-        <v>1.944</v>
+        <v>1.778</v>
       </c>
       <c r="H37" t="n">
-        <v>0.222</v>
+        <v>0.056</v>
       </c>
       <c r="I37" t="n">
-        <v>0.429</v>
+        <v>0.571</v>
       </c>
       <c r="J37" t="n">
-        <v>-0.3</v>
+        <v>0.3</v>
       </c>
       <c r="K37" t="n">
-        <v>-2.253</v>
+        <v>-3.02</v>
       </c>
       <c r="L37" t="n">
-        <v>-8.119999999999999</v>
+        <v>-6.38</v>
       </c>
       <c r="M37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2311,39 +2311,39 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45172</v>
+        <v>45156</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Middle Island Country Club - Oak and Spruce</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E38" t="n">
+        <v>4</v>
+      </c>
+      <c r="F38" t="n">
         <v>6</v>
       </c>
-      <c r="F38" t="n">
-        <v>8</v>
-      </c>
       <c r="G38" t="n">
-        <v>2.056</v>
+        <v>1.944</v>
       </c>
       <c r="H38" t="n">
-        <v>0.333</v>
+        <v>0.222</v>
       </c>
       <c r="I38" t="n">
-        <v>0.571</v>
+        <v>0.429</v>
       </c>
       <c r="J38" t="n">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="K38" t="n">
-        <v>-1.498</v>
+        <v>-2.253</v>
       </c>
       <c r="L38" t="n">
-        <v>-9.279999999999999</v>
+        <v>-8.119999999999999</v>
       </c>
       <c r="M38" t="n">
         <v>1</v>
@@ -2361,39 +2361,39 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45434</v>
+        <v>45172</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E39" t="n">
         <v>6</v>
       </c>
       <c r="F39" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G39" t="n">
-        <v>2.111</v>
+        <v>2.056</v>
       </c>
       <c r="H39" t="n">
         <v>0.333</v>
       </c>
       <c r="I39" t="n">
-        <v>0.214</v>
+        <v>0.571</v>
       </c>
       <c r="J39" t="n">
-        <v>-1.2</v>
+        <v>0.3</v>
       </c>
       <c r="K39" t="n">
-        <v>-2.471</v>
+        <v>-1.498</v>
       </c>
       <c r="L39" t="n">
-        <v>-10.28</v>
+        <v>-9.279999999999999</v>
       </c>
       <c r="M39" t="n">
         <v>1</v>
@@ -2411,7 +2411,7 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45440</v>
+        <v>45434</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -2419,38 +2419,38 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F40" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G40" t="n">
-        <v>1.833</v>
+        <v>2.111</v>
       </c>
       <c r="H40" t="n">
-        <v>0.111</v>
+        <v>0.333</v>
       </c>
       <c r="I40" t="n">
-        <v>0.571</v>
+        <v>0.214</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="K40" t="n">
-        <v>-5.711</v>
+        <v>-2.471</v>
       </c>
       <c r="L40" t="n">
-        <v>-6.96</v>
+        <v>-10.28</v>
       </c>
       <c r="M40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2461,46 +2461,46 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45443</v>
+        <v>45440</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G41" t="n">
-        <v>1.944</v>
+        <v>1.833</v>
       </c>
       <c r="H41" t="n">
-        <v>0.333</v>
+        <v>0.111</v>
       </c>
       <c r="I41" t="n">
-        <v>0.286</v>
+        <v>0.571</v>
       </c>
       <c r="J41" t="n">
-        <v>-0.9</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>-1.498</v>
+        <v>-5.711</v>
       </c>
       <c r="L41" t="n">
-        <v>-7.28</v>
+        <v>-6.96</v>
       </c>
       <c r="M41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2511,39 +2511,39 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45453</v>
+        <v>45443</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Willow Creek Hamlet Course</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D42" t="n">
         <v>35</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G42" t="n">
         <v>1.944</v>
       </c>
       <c r="H42" t="n">
-        <v>0.167</v>
+        <v>0.333</v>
       </c>
       <c r="I42" t="n">
-        <v>0.357</v>
+        <v>0.286</v>
       </c>
       <c r="J42" t="n">
-        <v>-0.45</v>
+        <v>-0.9</v>
       </c>
       <c r="K42" t="n">
-        <v>-5.437</v>
+        <v>-1.498</v>
       </c>
       <c r="L42" t="n">
-        <v>-8.539999999999999</v>
+        <v>-7.28</v>
       </c>
       <c r="M42" t="n">
         <v>1</v>
@@ -2561,42 +2561,42 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45465</v>
+        <v>45453</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Wind Watch Hamlet Course</t>
+          <t>Willow Creek Hamlet Course</t>
         </is>
       </c>
       <c r="D43" t="n">
         <v>35</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G43" t="n">
         <v>1.944</v>
       </c>
       <c r="H43" t="n">
-        <v>0.111</v>
+        <v>0.167</v>
       </c>
       <c r="I43" t="n">
-        <v>0.214</v>
+        <v>0.357</v>
       </c>
       <c r="J43" t="n">
-        <v>-1.2</v>
+        <v>-0.45</v>
       </c>
       <c r="K43" t="n">
-        <v>-5.476</v>
+        <v>-5.437</v>
       </c>
       <c r="L43" t="n">
-        <v>-8.960000000000001</v>
+        <v>-8.539999999999999</v>
       </c>
       <c r="M43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45466</v>
+        <v>45465</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bethpage Red</t>
+          <t>Wind Watch Hamlet Course</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="n">
+        <v>3</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1.944</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.214</v>
+      </c>
+      <c r="J44" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="K44" t="n">
+        <v>-5.476</v>
+      </c>
+      <c r="L44" t="n">
+        <v>-8.960000000000001</v>
+      </c>
+      <c r="M44" t="n">
         <v>4</v>
       </c>
-      <c r="F44" t="n">
-        <v>7</v>
-      </c>
-      <c r="G44" t="n">
-        <v>1.667</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0.222</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J44" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" t="n">
-        <v>-1.818</v>
-      </c>
-      <c r="L44" t="n">
-        <v>-3.12</v>
-      </c>
-      <c r="M44" t="n">
-        <v>2</v>
-      </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2661,46 +2661,46 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45467</v>
+        <v>45466</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Bethpage Red</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E45" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F45" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G45" t="n">
-        <v>1.833</v>
+        <v>1.667</v>
       </c>
       <c r="H45" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="I45" t="n">
         <v>0.5</v>
       </c>
-      <c r="I45" t="n">
-        <v>0.429</v>
-      </c>
       <c r="J45" t="n">
-        <v>-0.3</v>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>-0.976</v>
+        <v>-1.818</v>
       </c>
       <c r="L45" t="n">
-        <v>-4.02</v>
+        <v>-3.12</v>
       </c>
       <c r="M45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45475</v>
+        <v>45467</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -2719,31 +2719,31 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E46" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F46" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G46" t="n">
-        <v>1.611</v>
+        <v>1.833</v>
       </c>
       <c r="H46" t="n">
-        <v>0.444</v>
+        <v>0.5</v>
       </c>
       <c r="I46" t="n">
-        <v>0.571</v>
+        <v>0.429</v>
       </c>
       <c r="J46" t="n">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="K46" t="n">
-        <v>-0.253</v>
+        <v>-0.976</v>
       </c>
       <c r="L46" t="n">
-        <v>-0.44</v>
+        <v>-4.02</v>
       </c>
       <c r="M46" t="n">
         <v>3</v>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45480</v>
+        <v>45475</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Bethpage Red</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E47" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F47" t="n">
         <v>8</v>
       </c>
       <c r="G47" t="n">
-        <v>1.667</v>
+        <v>1.611</v>
       </c>
       <c r="H47" t="n">
-        <v>0.111</v>
+        <v>0.444</v>
       </c>
       <c r="I47" t="n">
         <v>0.571</v>
@@ -2790,17 +2790,17 @@
         <v>0.3</v>
       </c>
       <c r="K47" t="n">
-        <v>-2.422</v>
+        <v>-0.253</v>
       </c>
       <c r="L47" t="n">
-        <v>-3.96</v>
+        <v>-0.44</v>
       </c>
       <c r="M47" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -2811,46 +2811,46 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45487</v>
+        <v>45480</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Red</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E48" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G48" t="n">
-        <v>1.611</v>
+        <v>1.667</v>
       </c>
       <c r="H48" t="n">
-        <v>0.333</v>
+        <v>0.111</v>
       </c>
       <c r="I48" t="n">
-        <v>0.214</v>
+        <v>0.571</v>
       </c>
       <c r="J48" t="n">
-        <v>-1.2</v>
+        <v>0.3</v>
       </c>
       <c r="K48" t="n">
-        <v>-1.578</v>
+        <v>-2.422</v>
       </c>
       <c r="L48" t="n">
-        <v>-1.28</v>
+        <v>-3.96</v>
       </c>
       <c r="M48" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2861,39 +2861,39 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45492</v>
+        <v>45487</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D49" t="n">
         <v>29</v>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F49" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G49" t="n">
         <v>1.611</v>
       </c>
       <c r="H49" t="n">
-        <v>0.278</v>
+        <v>0.333</v>
       </c>
       <c r="I49" t="n">
-        <v>0.571</v>
+        <v>0.214</v>
       </c>
       <c r="J49" t="n">
-        <v>0.15</v>
+        <v>-1.2</v>
       </c>
       <c r="K49" t="n">
-        <v>-3.1</v>
+        <v>-1.578</v>
       </c>
       <c r="L49" t="n">
-        <v>-1.7</v>
+        <v>-1.28</v>
       </c>
       <c r="M49" t="n">
         <v>2</v>
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>45496</v>
+        <v>45492</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -2919,31 +2919,31 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F50" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G50" t="n">
-        <v>1.5</v>
+        <v>1.611</v>
       </c>
       <c r="H50" t="n">
-        <v>0.167</v>
+        <v>0.278</v>
       </c>
       <c r="I50" t="n">
-        <v>0.643</v>
+        <v>0.571</v>
       </c>
       <c r="J50" t="n">
-        <v>0.45</v>
+        <v>0.15</v>
       </c>
       <c r="K50" t="n">
-        <v>-4.1</v>
+        <v>-3.1</v>
       </c>
       <c r="L50" t="n">
-        <v>-0.54</v>
+        <v>-1.7</v>
       </c>
       <c r="M50" t="n">
         <v>2</v>
@@ -2961,39 +2961,39 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>45502</v>
+        <v>45496</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F51" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G51" t="n">
-        <v>1.611</v>
+        <v>1.5</v>
       </c>
       <c r="H51" t="n">
-        <v>0.222</v>
+        <v>0.167</v>
       </c>
       <c r="I51" t="n">
-        <v>0.429</v>
+        <v>0.643</v>
       </c>
       <c r="J51" t="n">
-        <v>-0.3</v>
+        <v>0.45</v>
       </c>
       <c r="K51" t="n">
-        <v>-3.578</v>
+        <v>-4.1</v>
       </c>
       <c r="L51" t="n">
-        <v>-2.12</v>
+        <v>-0.54</v>
       </c>
       <c r="M51" t="n">
         <v>2</v>
@@ -3011,15 +3011,15 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>45514</v>
+        <v>45502</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E52" t="n">
         <v>4</v>
@@ -3028,7 +3028,7 @@
         <v>6</v>
       </c>
       <c r="G52" t="n">
-        <v>1.722</v>
+        <v>1.611</v>
       </c>
       <c r="H52" t="n">
         <v>0.222</v>
@@ -3037,13 +3037,13 @@
         <v>0.429</v>
       </c>
       <c r="J52" t="n">
-        <v>-0.45</v>
+        <v>-0.3</v>
       </c>
       <c r="K52" t="n">
-        <v>-3.6</v>
+        <v>-3.578</v>
       </c>
       <c r="L52" t="n">
-        <v>-4.12</v>
+        <v>-2.12</v>
       </c>
       <c r="M52" t="n">
         <v>2</v>
@@ -3061,46 +3061,46 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>45535</v>
+        <v>45514</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F53" t="n">
         <v>6</v>
       </c>
       <c r="G53" t="n">
-        <v>1.778</v>
+        <v>1.722</v>
       </c>
       <c r="H53" t="n">
-        <v>0.167</v>
+        <v>0.222</v>
       </c>
       <c r="I53" t="n">
         <v>0.429</v>
       </c>
       <c r="J53" t="n">
-        <v>-0.3</v>
+        <v>-0.45</v>
       </c>
       <c r="K53" t="n">
-        <v>-5.433</v>
+        <v>-3.6</v>
       </c>
       <c r="L53" t="n">
-        <v>-5.54</v>
+        <v>-4.12</v>
       </c>
       <c r="M53" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3111,46 +3111,46 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>45570</v>
+        <v>45535</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E54" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F54" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G54" t="n">
-        <v>1.611</v>
+        <v>1.778</v>
       </c>
       <c r="H54" t="n">
-        <v>0.278</v>
+        <v>0.167</v>
       </c>
       <c r="I54" t="n">
-        <v>0.357</v>
+        <v>0.429</v>
       </c>
       <c r="J54" t="n">
-        <v>-0.6</v>
+        <v>-0.3</v>
       </c>
       <c r="K54" t="n">
-        <v>-3.676</v>
+        <v>-5.433</v>
       </c>
       <c r="L54" t="n">
-        <v>-2.12</v>
+        <v>-5.54</v>
       </c>
       <c r="M54" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3161,11 +3161,11 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45580</v>
+        <v>45570</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Sebonack Golf Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3175,7 +3175,7 @@
         <v>5</v>
       </c>
       <c r="F55" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G55" t="n">
         <v>1.611</v>
@@ -3184,16 +3184,16 @@
         <v>0.278</v>
       </c>
       <c r="I55" t="n">
-        <v>0.429</v>
+        <v>0.357</v>
       </c>
       <c r="J55" t="n">
-        <v>-0.3</v>
+        <v>-0.6</v>
       </c>
       <c r="K55" t="n">
-        <v>-3.789</v>
+        <v>-3.676</v>
       </c>
       <c r="L55" t="n">
-        <v>-1.7</v>
+        <v>-2.12</v>
       </c>
       <c r="M55" t="n">
         <v>2</v>
@@ -3211,46 +3211,46 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>45649</v>
+        <v>45580</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Ka'anapali Golf Resort Royal Course</t>
+          <t>Sebonack Golf Club</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E56" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F56" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G56" t="n">
-        <v>1.944</v>
+        <v>1.611</v>
       </c>
       <c r="H56" t="n">
-        <v>0.056</v>
+        <v>0.278</v>
       </c>
       <c r="I56" t="n">
-        <v>0.357</v>
+        <v>0.429</v>
       </c>
       <c r="J56" t="n">
-        <v>-0.6</v>
+        <v>-0.3</v>
       </c>
       <c r="K56" t="n">
-        <v>-4.167</v>
+        <v>-3.789</v>
       </c>
       <c r="L56" t="n">
-        <v>-9.380000000000001</v>
+        <v>-1.7</v>
       </c>
       <c r="M56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3261,46 +3261,46 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>45653</v>
+        <v>45649</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Wailea Golf Club Gold Course</t>
+          <t>Ka'anapali Golf Resort Royal Course</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
         <v>5</v>
       </c>
-      <c r="F57" t="n">
-        <v>3</v>
-      </c>
       <c r="G57" t="n">
-        <v>1.722</v>
+        <v>1.944</v>
       </c>
       <c r="H57" t="n">
-        <v>0.278</v>
+        <v>0.056</v>
       </c>
       <c r="I57" t="n">
-        <v>0.214</v>
+        <v>0.357</v>
       </c>
       <c r="J57" t="n">
-        <v>0.3</v>
+        <v>-0.6</v>
       </c>
       <c r="K57" t="n">
-        <v>-1.651</v>
+        <v>-4.167</v>
       </c>
       <c r="L57" t="n">
-        <v>-3.7</v>
+        <v>-9.380000000000001</v>
       </c>
       <c r="M57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3311,46 +3311,46 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>45655</v>
+        <v>45653</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Wailea Golf Club Emerald Course</t>
+          <t>Wailea Golf Club Gold Course</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F58" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="G58" t="n">
-        <v>1.889</v>
+        <v>1.722</v>
       </c>
       <c r="H58" t="n">
-        <v>0.333</v>
+        <v>0.278</v>
       </c>
       <c r="I58" t="n">
-        <v>0.786</v>
+        <v>0.214</v>
       </c>
       <c r="J58" t="n">
-        <v>1.2</v>
+        <v>0.3</v>
       </c>
       <c r="K58" t="n">
-        <v>-1.556</v>
+        <v>-1.651</v>
       </c>
       <c r="L58" t="n">
-        <v>-6.28</v>
+        <v>-3.7</v>
       </c>
       <c r="M58" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3361,46 +3361,46 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>45735</v>
+        <v>45655</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Wailea Golf Club Emerald Course</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E59" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F59" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G59" t="n">
-        <v>1.722</v>
+        <v>1.889</v>
       </c>
       <c r="H59" t="n">
-        <v>0.556</v>
+        <v>0.333</v>
       </c>
       <c r="I59" t="n">
-        <v>0.5</v>
+        <v>0.786</v>
       </c>
       <c r="J59" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K59" t="n">
+        <v>-1.556</v>
+      </c>
+      <c r="L59" t="n">
+        <v>-6.28</v>
+      </c>
+      <c r="M59" t="n">
         <v>0</v>
       </c>
-      <c r="K59" t="n">
-        <v>-0.676</v>
-      </c>
-      <c r="L59" t="n">
-        <v>-1.6</v>
-      </c>
-      <c r="M59" t="n">
-        <v>3</v>
-      </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -3411,39 +3411,39 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>45829</v>
+        <v>45735</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E60" t="n">
+        <v>10</v>
+      </c>
+      <c r="F60" t="n">
         <v>7</v>
       </c>
-      <c r="F60" t="n">
-        <v>9</v>
-      </c>
       <c r="G60" t="n">
-        <v>1.556</v>
+        <v>1.722</v>
       </c>
       <c r="H60" t="n">
-        <v>0.389</v>
+        <v>0.556</v>
       </c>
       <c r="I60" t="n">
-        <v>0.643</v>
+        <v>0.5</v>
       </c>
       <c r="J60" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="K60" t="n">
-        <v>-1.45</v>
+        <v>-0.676</v>
       </c>
       <c r="L60" t="n">
-        <v>0.14</v>
+        <v>-1.6</v>
       </c>
       <c r="M60" t="n">
         <v>3</v>
@@ -3461,39 +3461,39 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45831</v>
+        <v>45829</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E61" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F61" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G61" t="n">
-        <v>1.778</v>
+        <v>1.556</v>
       </c>
       <c r="H61" t="n">
-        <v>0.444</v>
+        <v>0.389</v>
       </c>
       <c r="I61" t="n">
-        <v>0.571</v>
+        <v>0.643</v>
       </c>
       <c r="J61" t="n">
-        <v>0.3</v>
+        <v>0.45</v>
       </c>
       <c r="K61" t="n">
-        <v>0.247</v>
+        <v>-1.45</v>
       </c>
       <c r="L61" t="n">
-        <v>-3.02</v>
+        <v>0.14</v>
       </c>
       <c r="M61" t="n">
         <v>3</v>
@@ -3511,11 +3511,11 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45844</v>
+        <v>45831</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3525,7 +3525,7 @@
         <v>8</v>
       </c>
       <c r="F62" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G62" t="n">
         <v>1.778</v>
@@ -3534,16 +3534,16 @@
         <v>0.444</v>
       </c>
       <c r="I62" t="n">
-        <v>0.5</v>
+        <v>0.571</v>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="K62" t="n">
-        <v>-1.596</v>
+        <v>0.247</v>
       </c>
       <c r="L62" t="n">
-        <v>-3.44</v>
+        <v>-3.02</v>
       </c>
       <c r="M62" t="n">
         <v>3</v>
@@ -3561,7 +3561,7 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>45857</v>
+        <v>45844</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -3569,31 +3569,31 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E63" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F63" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G63" t="n">
-        <v>1.833</v>
+        <v>1.778</v>
       </c>
       <c r="H63" t="n">
-        <v>0.611</v>
+        <v>0.444</v>
       </c>
       <c r="I63" t="n">
-        <v>0.571</v>
+        <v>0.5</v>
       </c>
       <c r="J63" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="K63" t="n">
-        <v>0.904</v>
+        <v>-1.596</v>
       </c>
       <c r="L63" t="n">
-        <v>-3.18</v>
+        <v>-3.44</v>
       </c>
       <c r="M63" t="n">
         <v>3</v>
@@ -3611,46 +3611,46 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45868</v>
+        <v>45857</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Bethpage Red</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E64" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F64" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G64" t="n">
-        <v>1.611</v>
+        <v>1.833</v>
       </c>
       <c r="H64" t="n">
-        <v>0.222</v>
+        <v>0.611</v>
       </c>
       <c r="I64" t="n">
-        <v>0.5</v>
+        <v>0.571</v>
       </c>
       <c r="J64" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K64" t="n">
-        <v>-1.342</v>
+        <v>0.904</v>
       </c>
       <c r="L64" t="n">
-        <v>-2.12</v>
+        <v>-3.18</v>
       </c>
       <c r="M64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -3661,46 +3661,46 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>45886</v>
+        <v>45868</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Spring Lake Thunderbird</t>
+          <t>Bethpage Red</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E65" t="n">
         <v>4</v>
       </c>
       <c r="F65" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G65" t="n">
-        <v>1.667</v>
+        <v>1.611</v>
       </c>
       <c r="H65" t="n">
         <v>0.222</v>
       </c>
       <c r="I65" t="n">
-        <v>0.786</v>
+        <v>0.5</v>
       </c>
       <c r="J65" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="K65" t="n">
-        <v>-3.573</v>
+        <v>-1.342</v>
       </c>
       <c r="L65" t="n">
-        <v>-3.12</v>
+        <v>-2.12</v>
       </c>
       <c r="M65" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>45892</v>
+        <v>45886</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -3719,38 +3719,38 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E66" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F66" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G66" t="n">
-        <v>1.778</v>
+        <v>1.667</v>
       </c>
       <c r="H66" t="n">
-        <v>0.278</v>
+        <v>0.222</v>
       </c>
       <c r="I66" t="n">
-        <v>0.429</v>
+        <v>0.786</v>
       </c>
       <c r="J66" t="n">
-        <v>-0.3</v>
+        <v>1.2</v>
       </c>
       <c r="K66" t="n">
-        <v>-3.153</v>
+        <v>-3.573</v>
       </c>
       <c r="L66" t="n">
-        <v>-4.7</v>
+        <v>-3.12</v>
       </c>
       <c r="M66" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -3761,46 +3761,46 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>45894</v>
+        <v>45892</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Willow Creek Hamlet Course</t>
+          <t>Spring Lake Thunderbird</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E67" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F67" t="n">
         <v>6</v>
       </c>
       <c r="G67" t="n">
-        <v>2.111</v>
+        <v>1.778</v>
       </c>
       <c r="H67" t="n">
-        <v>0.056</v>
+        <v>0.278</v>
       </c>
       <c r="I67" t="n">
         <v>0.429</v>
       </c>
       <c r="J67" t="n">
-        <v>-0.15</v>
+        <v>-0.3</v>
       </c>
       <c r="K67" t="n">
-        <v>-5.517</v>
+        <v>-3.153</v>
       </c>
       <c r="L67" t="n">
-        <v>-12.38</v>
+        <v>-4.7</v>
       </c>
       <c r="M67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3811,42 +3811,42 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>45897</v>
+        <v>45894</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Spring Lake Thunderbird</t>
+          <t>Willow Creek Hamlet Course</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E68" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F68" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G68" t="n">
-        <v>1.722</v>
+        <v>2.111</v>
       </c>
       <c r="H68" t="n">
-        <v>0.222</v>
+        <v>0.056</v>
       </c>
       <c r="I68" t="n">
-        <v>0.214</v>
+        <v>0.429</v>
       </c>
       <c r="J68" t="n">
-        <v>-1.2</v>
+        <v>-0.15</v>
       </c>
       <c r="K68" t="n">
-        <v>-5.733</v>
+        <v>-5.517</v>
       </c>
       <c r="L68" t="n">
-        <v>-4.12</v>
+        <v>-12.38</v>
       </c>
       <c r="M68" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
@@ -3861,27 +3861,27 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>45941</v>
+        <v>45897</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Wind Watch Hamlet Course</t>
+          <t>Spring Lake Thunderbird</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F69" t="n">
         <v>3</v>
       </c>
       <c r="G69" t="n">
-        <v>1.667</v>
+        <v>1.722</v>
       </c>
       <c r="H69" t="n">
-        <v>0.056</v>
+        <v>0.222</v>
       </c>
       <c r="I69" t="n">
         <v>0.214</v>
@@ -3890,10 +3890,10 @@
         <v>-1.2</v>
       </c>
       <c r="K69" t="n">
-        <v>-5.522</v>
+        <v>-5.733</v>
       </c>
       <c r="L69" t="n">
-        <v>-4.38</v>
+        <v>-4.12</v>
       </c>
       <c r="M69" t="n">
         <v>4</v>
@@ -3911,46 +3911,46 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>46160</v>
+        <v>45941</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Wind Watch Hamlet Course</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E70" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F70" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G70" t="n">
-        <v>1.889</v>
+        <v>1.667</v>
       </c>
       <c r="H70" t="n">
-        <v>0.444</v>
+        <v>0.056</v>
       </c>
       <c r="I70" t="n">
-        <v>0.357</v>
+        <v>0.214</v>
       </c>
       <c r="J70" t="n">
-        <v>-0.6</v>
+        <v>-1.2</v>
       </c>
       <c r="K70" t="n">
-        <v>-0.173</v>
+        <v>-5.522</v>
       </c>
       <c r="L70" t="n">
-        <v>-5.44</v>
+        <v>-4.38</v>
       </c>
       <c r="M70" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3961,46 +3961,46 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>46164</v>
+        <v>46160</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E71" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F71" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G71" t="n">
-        <v>1.722</v>
+        <v>1.889</v>
       </c>
       <c r="H71" t="n">
-        <v>0.111</v>
+        <v>0.444</v>
       </c>
       <c r="I71" t="n">
-        <v>0.643</v>
+        <v>0.357</v>
       </c>
       <c r="J71" t="n">
-        <v>0.45</v>
+        <v>-0.6</v>
       </c>
       <c r="K71" t="n">
-        <v>-3.95</v>
+        <v>-0.173</v>
       </c>
       <c r="L71" t="n">
-        <v>-4.96</v>
+        <v>-5.44</v>
       </c>
       <c r="M71" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -4011,44 +4011,94 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
+        <v>46164</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Brentwood Country Club</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>31</v>
+      </c>
+      <c r="E72" t="n">
+        <v>2</v>
+      </c>
+      <c r="F72" t="n">
+        <v>9</v>
+      </c>
+      <c r="G72" t="n">
+        <v>1.722</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K72" t="n">
+        <v>-3.95</v>
+      </c>
+      <c r="L72" t="n">
+        <v>-4.96</v>
+      </c>
+      <c r="M72" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>All Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
         <v>46173</v>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>Bethpage Green</t>
         </is>
       </c>
-      <c r="D72" t="n">
+      <c r="D73" t="n">
         <v>35</v>
       </c>
-      <c r="E72" t="n">
+      <c r="E73" t="n">
         <v>5</v>
       </c>
-      <c r="F72" t="n">
+      <c r="F73" t="n">
         <v>5</v>
       </c>
-      <c r="G72" t="n">
+      <c r="G73" t="n">
         <v>1.944</v>
       </c>
-      <c r="H72" t="n">
+      <c r="H73" t="n">
         <v>0.278</v>
       </c>
-      <c r="I72" t="n">
+      <c r="I73" t="n">
         <v>0.357</v>
       </c>
-      <c r="J72" t="n">
+      <c r="J73" t="n">
         <v>-0.6</v>
       </c>
-      <c r="K72" t="n">
+      <c r="K73" t="n">
         <v>-3.256</v>
       </c>
-      <c r="L72" t="n">
+      <c r="L73" t="n">
         <v>-7.7</v>
       </c>
-      <c r="M72" t="n">
+      <c r="M73" t="n">
         <v>1</v>
       </c>
-      <c r="N72" t="inlineStr">
+      <c r="N73" t="inlineStr">
         <is>
           <t>Ball Striker</t>
         </is>

</xml_diff>

<commit_message>
Update golf analytics and data files with revised metrics and recommendations
- Adjusted cluster averages for Ryan and Tyler in the Golf Analytics notebook.
- Updated recommended club and distance ranges based on new analysis.
- Changed course name from "Bethpage Black" to "Baiting Hollow" in multiple instances.
- Refined recommendations for tee shots and approach strategies.
- Updated various Excel files including 'Golf Stats', 'club_ranges', 'club_selector', 'clustered_rounds', 'clutch_score_analysis', 'golf_recommendations', and 'strokes_gained_summary' with new data.
</commit_message>
<xml_diff>
--- a/clustered_rounds.xlsx
+++ b/clustered_rounds.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N76"/>
+  <dimension ref="A1:N78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1546,11 +1546,11 @@
         <v>-9.380000000000001</v>
       </c>
       <c r="M22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Off Day</t>
         </is>
       </c>
     </row>
@@ -1596,11 +1596,11 @@
         <v>-8.380000000000001</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Off Day</t>
         </is>
       </c>
     </row>
@@ -1646,11 +1646,11 @@
         <v>-9.119999999999999</v>
       </c>
       <c r="M24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Off Day</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1696,11 +1696,11 @@
         <v>-15.96</v>
       </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Off Day</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -1746,11 +1746,11 @@
         <v>-18.96</v>
       </c>
       <c r="M26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -1796,11 +1796,11 @@
         <v>-15.54</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Off Day</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -1846,11 +1846,11 @@
         <v>-14.12</v>
       </c>
       <c r="M28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Off Day</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -1896,54 +1896,54 @@
         <v>-7.96</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Off Day</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45048</v>
+        <v>46211</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Baiting Hollow</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>2.556</v>
       </c>
       <c r="H30" t="n">
-        <v>0.167</v>
+        <v>0.111</v>
       </c>
       <c r="I30" t="n">
-        <v>0.643</v>
+        <v>0.429</v>
       </c>
       <c r="J30" t="n">
-        <v>0.6</v>
+        <v>-0.3</v>
       </c>
       <c r="K30" t="n">
-        <v>-4.753</v>
+        <v>-6.387</v>
       </c>
       <c r="L30" t="n">
-        <v>-9.539999999999999</v>
+        <v>-19.96</v>
       </c>
       <c r="M30" t="n">
         <v>0</v>
@@ -1961,46 +1961,46 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45050</v>
+        <v>45048</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G31" t="n">
-        <v>2.056</v>
+        <v>2</v>
       </c>
       <c r="H31" t="n">
-        <v>0.222</v>
+        <v>0.167</v>
       </c>
       <c r="I31" t="n">
-        <v>0.5</v>
+        <v>0.643</v>
       </c>
       <c r="J31" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K31" t="n">
+        <v>-4.753</v>
+      </c>
+      <c r="L31" t="n">
+        <v>-9.539999999999999</v>
+      </c>
+      <c r="M31" t="n">
         <v>0</v>
       </c>
-      <c r="K31" t="n">
-        <v>-4.418</v>
-      </c>
-      <c r="L31" t="n">
-        <v>-10.12</v>
-      </c>
-      <c r="M31" t="n">
-        <v>1</v>
-      </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45053</v>
+        <v>45050</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -2040,17 +2040,17 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>-3.498</v>
+        <v>-4.418</v>
       </c>
       <c r="L32" t="n">
         <v>-10.12</v>
       </c>
       <c r="M32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2065,42 +2065,42 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F33" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G33" t="n">
-        <v>2</v>
+        <v>2.056</v>
       </c>
       <c r="H33" t="n">
-        <v>0.111</v>
+        <v>0.222</v>
       </c>
       <c r="I33" t="n">
-        <v>0.429</v>
+        <v>0.5</v>
       </c>
       <c r="J33" t="n">
-        <v>-0.3</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>-5.631</v>
+        <v>-3.498</v>
       </c>
       <c r="L33" t="n">
-        <v>-9.960000000000001</v>
+        <v>-10.12</v>
       </c>
       <c r="M33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2111,15 +2111,15 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45084</v>
+        <v>45053</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E34" t="n">
         <v>2</v>
@@ -2128,7 +2128,7 @@
         <v>6</v>
       </c>
       <c r="G34" t="n">
-        <v>2.056</v>
+        <v>2</v>
       </c>
       <c r="H34" t="n">
         <v>0.111</v>
@@ -2140,17 +2140,17 @@
         <v>-0.3</v>
       </c>
       <c r="K34" t="n">
-        <v>-4.333</v>
+        <v>-5.631</v>
       </c>
       <c r="L34" t="n">
-        <v>-10.96</v>
+        <v>-9.960000000000001</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45114</v>
+        <v>45084</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -2169,38 +2169,38 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E35" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G35" t="n">
-        <v>1.778</v>
+        <v>2.056</v>
       </c>
       <c r="H35" t="n">
-        <v>0.278</v>
+        <v>0.111</v>
       </c>
       <c r="I35" t="n">
-        <v>0.214</v>
+        <v>0.429</v>
       </c>
       <c r="J35" t="n">
-        <v>-1.05</v>
+        <v>-0.3</v>
       </c>
       <c r="K35" t="n">
-        <v>-6.473</v>
+        <v>-4.333</v>
       </c>
       <c r="L35" t="n">
-        <v>-5.1</v>
+        <v>-10.96</v>
       </c>
       <c r="M35" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45136</v>
+        <v>45114</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -2219,38 +2219,38 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E36" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" t="n">
         <v>3</v>
       </c>
-      <c r="F36" t="n">
-        <v>6</v>
-      </c>
       <c r="G36" t="n">
-        <v>1.722</v>
+        <v>1.778</v>
       </c>
       <c r="H36" t="n">
-        <v>0.167</v>
+        <v>0.278</v>
       </c>
       <c r="I36" t="n">
-        <v>0.429</v>
+        <v>0.214</v>
       </c>
       <c r="J36" t="n">
-        <v>-0.15</v>
+        <v>-1.05</v>
       </c>
       <c r="K36" t="n">
-        <v>-0.2</v>
+        <v>-6.473</v>
       </c>
       <c r="L36" t="n">
-        <v>-0.6</v>
+        <v>-5.1</v>
       </c>
       <c r="M36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -2261,39 +2261,39 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45137</v>
+        <v>45136</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G37" t="n">
-        <v>1.778</v>
+        <v>1.722</v>
       </c>
       <c r="H37" t="n">
-        <v>0.222</v>
+        <v>0.167</v>
       </c>
       <c r="I37" t="n">
-        <v>0.286</v>
+        <v>0.429</v>
       </c>
       <c r="J37" t="n">
-        <v>-0.9</v>
+        <v>-0.15</v>
       </c>
       <c r="K37" t="n">
-        <v>-4.631</v>
+        <v>-0.2</v>
       </c>
       <c r="L37" t="n">
-        <v>-5.12</v>
+        <v>-0.6</v>
       </c>
       <c r="M37" t="n">
         <v>4</v>
@@ -2311,7 +2311,7 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45143</v>
+        <v>45137</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -2319,38 +2319,38 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="E38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G38" t="n">
-        <v>2.167</v>
+        <v>1.778</v>
       </c>
       <c r="H38" t="n">
-        <v>0.278</v>
+        <v>0.222</v>
       </c>
       <c r="I38" t="n">
-        <v>0.429</v>
+        <v>0.286</v>
       </c>
       <c r="J38" t="n">
-        <v>-0.3</v>
+        <v>-0.9</v>
       </c>
       <c r="K38" t="n">
-        <v>-2.051</v>
+        <v>-4.631</v>
       </c>
       <c r="L38" t="n">
-        <v>-11.7</v>
+        <v>-5.12</v>
       </c>
       <c r="M38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -2361,39 +2361,39 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45144</v>
+        <v>45143</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Bethpage Black</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F39" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G39" t="n">
-        <v>1.778</v>
+        <v>2.167</v>
       </c>
       <c r="H39" t="n">
-        <v>0.056</v>
+        <v>0.278</v>
       </c>
       <c r="I39" t="n">
-        <v>0.571</v>
+        <v>0.429</v>
       </c>
       <c r="J39" t="n">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="K39" t="n">
-        <v>-3.02</v>
+        <v>-2.051</v>
       </c>
       <c r="L39" t="n">
-        <v>-6.38</v>
+        <v>-11.7</v>
       </c>
       <c r="M39" t="n">
         <v>0</v>
@@ -2411,39 +2411,39 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45156</v>
+        <v>45144</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Middle Island Country Club - Oak and Spruce</t>
+          <t>Bethpage Black</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G40" t="n">
-        <v>1.944</v>
+        <v>1.778</v>
       </c>
       <c r="H40" t="n">
-        <v>0.222</v>
+        <v>0.056</v>
       </c>
       <c r="I40" t="n">
-        <v>0.429</v>
+        <v>0.571</v>
       </c>
       <c r="J40" t="n">
-        <v>-0.3</v>
+        <v>0.3</v>
       </c>
       <c r="K40" t="n">
-        <v>-2.253</v>
+        <v>-3.02</v>
       </c>
       <c r="L40" t="n">
-        <v>-8.119999999999999</v>
+        <v>-6.38</v>
       </c>
       <c r="M40" t="n">
         <v>1</v>
@@ -2461,46 +2461,46 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45172</v>
+        <v>45156</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Middle Island Country Club - Oak and Spruce</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E41" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" t="n">
         <v>6</v>
       </c>
-      <c r="F41" t="n">
-        <v>8</v>
-      </c>
       <c r="G41" t="n">
-        <v>2.056</v>
+        <v>1.944</v>
       </c>
       <c r="H41" t="n">
-        <v>0.333</v>
+        <v>0.222</v>
       </c>
       <c r="I41" t="n">
-        <v>0.571</v>
+        <v>0.429</v>
       </c>
       <c r="J41" t="n">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="K41" t="n">
-        <v>-1.498</v>
+        <v>-2.253</v>
       </c>
       <c r="L41" t="n">
-        <v>-9.279999999999999</v>
+        <v>-8.119999999999999</v>
       </c>
       <c r="M41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2511,46 +2511,46 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45434</v>
+        <v>45172</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E42" t="n">
         <v>6</v>
       </c>
       <c r="F42" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G42" t="n">
-        <v>2.111</v>
+        <v>2.056</v>
       </c>
       <c r="H42" t="n">
         <v>0.333</v>
       </c>
       <c r="I42" t="n">
-        <v>0.214</v>
+        <v>0.571</v>
       </c>
       <c r="J42" t="n">
-        <v>-1.2</v>
+        <v>0.3</v>
       </c>
       <c r="K42" t="n">
-        <v>-2.471</v>
+        <v>-1.498</v>
       </c>
       <c r="L42" t="n">
-        <v>-10.28</v>
+        <v>-9.279999999999999</v>
       </c>
       <c r="M42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45440</v>
+        <v>45434</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -2569,31 +2569,31 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F43" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G43" t="n">
-        <v>1.833</v>
+        <v>2.111</v>
       </c>
       <c r="H43" t="n">
-        <v>0.111</v>
+        <v>0.333</v>
       </c>
       <c r="I43" t="n">
-        <v>0.571</v>
+        <v>0.214</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="K43" t="n">
-        <v>-5.711</v>
+        <v>-2.471</v>
       </c>
       <c r="L43" t="n">
-        <v>-6.96</v>
+        <v>-10.28</v>
       </c>
       <c r="M43" t="n">
         <v>0</v>
@@ -2611,46 +2611,46 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45443</v>
+        <v>45440</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E44" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F44" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G44" t="n">
-        <v>1.944</v>
+        <v>1.833</v>
       </c>
       <c r="H44" t="n">
-        <v>0.333</v>
+        <v>0.111</v>
       </c>
       <c r="I44" t="n">
-        <v>0.286</v>
+        <v>0.571</v>
       </c>
       <c r="J44" t="n">
-        <v>-0.9</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>-1.498</v>
+        <v>-5.711</v>
       </c>
       <c r="L44" t="n">
-        <v>-7.28</v>
+        <v>-6.96</v>
       </c>
       <c r="M44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2661,46 +2661,46 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45453</v>
+        <v>45443</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Willow Creek Hamlet Course</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D45" t="n">
         <v>35</v>
       </c>
       <c r="E45" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G45" t="n">
         <v>1.944</v>
       </c>
       <c r="H45" t="n">
-        <v>0.167</v>
+        <v>0.333</v>
       </c>
       <c r="I45" t="n">
-        <v>0.357</v>
+        <v>0.286</v>
       </c>
       <c r="J45" t="n">
-        <v>-0.45</v>
+        <v>-0.9</v>
       </c>
       <c r="K45" t="n">
-        <v>-5.437</v>
+        <v>-1.498</v>
       </c>
       <c r="L45" t="n">
-        <v>-8.539999999999999</v>
+        <v>-7.28</v>
       </c>
       <c r="M45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2711,46 +2711,46 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45465</v>
+        <v>45453</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Wind Watch Hamlet Course</t>
+          <t>Willow Creek Hamlet Course</t>
         </is>
       </c>
       <c r="D46" t="n">
         <v>35</v>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G46" t="n">
         <v>1.944</v>
       </c>
       <c r="H46" t="n">
-        <v>0.111</v>
+        <v>0.167</v>
       </c>
       <c r="I46" t="n">
-        <v>0.214</v>
+        <v>0.357</v>
       </c>
       <c r="J46" t="n">
-        <v>-1.2</v>
+        <v>-0.45</v>
       </c>
       <c r="K46" t="n">
-        <v>-5.476</v>
+        <v>-5.437</v>
       </c>
       <c r="L46" t="n">
-        <v>-8.960000000000001</v>
+        <v>-8.539999999999999</v>
       </c>
       <c r="M46" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -2761,46 +2761,46 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45466</v>
+        <v>45465</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Bethpage Red</t>
+          <t>Wind Watch Hamlet Course</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G47" t="n">
-        <v>1.667</v>
+        <v>1.944</v>
       </c>
       <c r="H47" t="n">
-        <v>0.222</v>
+        <v>0.111</v>
       </c>
       <c r="I47" t="n">
-        <v>0.5</v>
+        <v>0.214</v>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="K47" t="n">
-        <v>-1.818</v>
+        <v>-5.476</v>
       </c>
       <c r="L47" t="n">
-        <v>-3.12</v>
+        <v>-8.960000000000001</v>
       </c>
       <c r="M47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -2811,46 +2811,46 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45467</v>
+        <v>45466</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Bethpage Red</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E48" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F48" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G48" t="n">
-        <v>1.833</v>
+        <v>1.667</v>
       </c>
       <c r="H48" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="I48" t="n">
         <v>0.5</v>
       </c>
-      <c r="I48" t="n">
-        <v>0.429</v>
-      </c>
       <c r="J48" t="n">
-        <v>-0.3</v>
+        <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>-0.976</v>
+        <v>-1.818</v>
       </c>
       <c r="L48" t="n">
-        <v>-4.02</v>
+        <v>-3.12</v>
       </c>
       <c r="M48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45475</v>
+        <v>45467</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -2869,38 +2869,38 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E49" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F49" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G49" t="n">
-        <v>1.611</v>
+        <v>1.833</v>
       </c>
       <c r="H49" t="n">
-        <v>0.444</v>
+        <v>0.5</v>
       </c>
       <c r="I49" t="n">
-        <v>0.571</v>
+        <v>0.429</v>
       </c>
       <c r="J49" t="n">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="K49" t="n">
-        <v>-0.253</v>
+        <v>-0.976</v>
       </c>
       <c r="L49" t="n">
-        <v>-0.44</v>
+        <v>-4.02</v>
       </c>
       <c r="M49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2911,27 +2911,27 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>45480</v>
+        <v>45475</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Bethpage Red</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E50" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F50" t="n">
         <v>8</v>
       </c>
       <c r="G50" t="n">
-        <v>1.667</v>
+        <v>1.611</v>
       </c>
       <c r="H50" t="n">
-        <v>0.111</v>
+        <v>0.444</v>
       </c>
       <c r="I50" t="n">
         <v>0.571</v>
@@ -2940,17 +2940,17 @@
         <v>0.3</v>
       </c>
       <c r="K50" t="n">
-        <v>-2.422</v>
+        <v>-0.253</v>
       </c>
       <c r="L50" t="n">
-        <v>-3.96</v>
+        <v>-0.44</v>
       </c>
       <c r="M50" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -2961,46 +2961,46 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>45487</v>
+        <v>45480</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Red</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E51" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F51" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G51" t="n">
-        <v>1.611</v>
+        <v>1.667</v>
       </c>
       <c r="H51" t="n">
-        <v>0.333</v>
+        <v>0.111</v>
       </c>
       <c r="I51" t="n">
-        <v>0.214</v>
+        <v>0.571</v>
       </c>
       <c r="J51" t="n">
-        <v>-1.2</v>
+        <v>0.3</v>
       </c>
       <c r="K51" t="n">
-        <v>-1.578</v>
+        <v>-2.422</v>
       </c>
       <c r="L51" t="n">
-        <v>-1.28</v>
+        <v>-3.96</v>
       </c>
       <c r="M51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3011,46 +3011,46 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>45492</v>
+        <v>45487</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D52" t="n">
         <v>29</v>
       </c>
       <c r="E52" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F52" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G52" t="n">
         <v>1.611</v>
       </c>
       <c r="H52" t="n">
-        <v>0.278</v>
+        <v>0.333</v>
       </c>
       <c r="I52" t="n">
-        <v>0.571</v>
+        <v>0.214</v>
       </c>
       <c r="J52" t="n">
-        <v>0.15</v>
+        <v>-1.2</v>
       </c>
       <c r="K52" t="n">
-        <v>-3.1</v>
+        <v>-1.578</v>
       </c>
       <c r="L52" t="n">
-        <v>-1.7</v>
+        <v>-1.28</v>
       </c>
       <c r="M52" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>45496</v>
+        <v>45492</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -3069,38 +3069,38 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E53" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F53" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G53" t="n">
-        <v>1.5</v>
+        <v>1.611</v>
       </c>
       <c r="H53" t="n">
-        <v>0.167</v>
+        <v>0.278</v>
       </c>
       <c r="I53" t="n">
-        <v>0.643</v>
+        <v>0.571</v>
       </c>
       <c r="J53" t="n">
-        <v>0.45</v>
+        <v>0.15</v>
       </c>
       <c r="K53" t="n">
-        <v>-4.1</v>
+        <v>-3.1</v>
       </c>
       <c r="L53" t="n">
-        <v>-0.54</v>
+        <v>-1.7</v>
       </c>
       <c r="M53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3111,46 +3111,46 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>45502</v>
+        <v>45496</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F54" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G54" t="n">
-        <v>1.611</v>
+        <v>1.5</v>
       </c>
       <c r="H54" t="n">
-        <v>0.222</v>
+        <v>0.167</v>
       </c>
       <c r="I54" t="n">
-        <v>0.429</v>
+        <v>0.643</v>
       </c>
       <c r="J54" t="n">
-        <v>-0.3</v>
+        <v>0.45</v>
       </c>
       <c r="K54" t="n">
-        <v>-3.578</v>
+        <v>-4.1</v>
       </c>
       <c r="L54" t="n">
-        <v>-2.12</v>
+        <v>-0.54</v>
       </c>
       <c r="M54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3161,15 +3161,15 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45514</v>
+        <v>45502</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E55" t="n">
         <v>4</v>
@@ -3178,7 +3178,7 @@
         <v>6</v>
       </c>
       <c r="G55" t="n">
-        <v>1.722</v>
+        <v>1.611</v>
       </c>
       <c r="H55" t="n">
         <v>0.222</v>
@@ -3187,20 +3187,20 @@
         <v>0.429</v>
       </c>
       <c r="J55" t="n">
-        <v>-0.45</v>
+        <v>-0.3</v>
       </c>
       <c r="K55" t="n">
-        <v>-3.6</v>
+        <v>-3.578</v>
       </c>
       <c r="L55" t="n">
-        <v>-4.12</v>
+        <v>-2.12</v>
       </c>
       <c r="M55" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3211,39 +3211,39 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>45535</v>
+        <v>45514</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Bethpage Yellow</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F56" t="n">
         <v>6</v>
       </c>
       <c r="G56" t="n">
-        <v>1.778</v>
+        <v>1.722</v>
       </c>
       <c r="H56" t="n">
-        <v>0.167</v>
+        <v>0.222</v>
       </c>
       <c r="I56" t="n">
         <v>0.429</v>
       </c>
       <c r="J56" t="n">
-        <v>-0.3</v>
+        <v>-0.45</v>
       </c>
       <c r="K56" t="n">
-        <v>-5.433</v>
+        <v>-3.6</v>
       </c>
       <c r="L56" t="n">
-        <v>-5.54</v>
+        <v>-4.12</v>
       </c>
       <c r="M56" t="n">
         <v>4</v>
@@ -3261,46 +3261,46 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>45570</v>
+        <v>45535</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Yellow</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E57" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F57" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G57" t="n">
-        <v>1.611</v>
+        <v>1.778</v>
       </c>
       <c r="H57" t="n">
-        <v>0.278</v>
+        <v>0.167</v>
       </c>
       <c r="I57" t="n">
-        <v>0.357</v>
+        <v>0.429</v>
       </c>
       <c r="J57" t="n">
-        <v>-0.6</v>
+        <v>-0.3</v>
       </c>
       <c r="K57" t="n">
-        <v>-3.676</v>
+        <v>-5.433</v>
       </c>
       <c r="L57" t="n">
-        <v>-2.12</v>
+        <v>-5.54</v>
       </c>
       <c r="M57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>45580</v>
+        <v>45570</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sebonack Golf Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3325,7 +3325,7 @@
         <v>5</v>
       </c>
       <c r="F58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G58" t="n">
         <v>1.611</v>
@@ -3334,23 +3334,23 @@
         <v>0.278</v>
       </c>
       <c r="I58" t="n">
-        <v>0.429</v>
+        <v>0.357</v>
       </c>
       <c r="J58" t="n">
-        <v>-0.3</v>
+        <v>-0.6</v>
       </c>
       <c r="K58" t="n">
-        <v>-3.789</v>
+        <v>-3.676</v>
       </c>
       <c r="L58" t="n">
-        <v>-1.7</v>
+        <v>-2.12</v>
       </c>
       <c r="M58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3361,42 +3361,42 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>45649</v>
+        <v>45580</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Ka'anapali Golf Resort Royal Course</t>
+          <t>Sebonack Golf Club</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F59" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G59" t="n">
-        <v>1.944</v>
+        <v>1.611</v>
       </c>
       <c r="H59" t="n">
-        <v>0.056</v>
+        <v>0.278</v>
       </c>
       <c r="I59" t="n">
-        <v>0.357</v>
+        <v>0.429</v>
       </c>
       <c r="J59" t="n">
-        <v>-0.6</v>
+        <v>-0.3</v>
       </c>
       <c r="K59" t="n">
-        <v>-4.167</v>
+        <v>-3.789</v>
       </c>
       <c r="L59" t="n">
-        <v>-9.380000000000001</v>
+        <v>-1.7</v>
       </c>
       <c r="M59" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
@@ -3411,46 +3411,46 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>45653</v>
+        <v>45649</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Wailea Golf Club Gold Course</t>
+          <t>Ka'anapali Golf Resort Royal Course</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" t="n">
         <v>5</v>
       </c>
-      <c r="F60" t="n">
-        <v>3</v>
-      </c>
       <c r="G60" t="n">
-        <v>1.722</v>
+        <v>1.944</v>
       </c>
       <c r="H60" t="n">
-        <v>0.278</v>
+        <v>0.056</v>
       </c>
       <c r="I60" t="n">
-        <v>0.214</v>
+        <v>0.357</v>
       </c>
       <c r="J60" t="n">
-        <v>0.3</v>
+        <v>-0.6</v>
       </c>
       <c r="K60" t="n">
-        <v>-1.651</v>
+        <v>-4.167</v>
       </c>
       <c r="L60" t="n">
-        <v>-3.7</v>
+        <v>-9.380000000000001</v>
       </c>
       <c r="M60" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -3461,46 +3461,46 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45655</v>
+        <v>45653</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Wailea Golf Club Emerald Course</t>
+          <t>Wailea Golf Club Gold Course</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F61" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="G61" t="n">
-        <v>1.889</v>
+        <v>1.722</v>
       </c>
       <c r="H61" t="n">
-        <v>0.333</v>
+        <v>0.278</v>
       </c>
       <c r="I61" t="n">
-        <v>0.786</v>
+        <v>0.214</v>
       </c>
       <c r="J61" t="n">
-        <v>1.2</v>
+        <v>0.3</v>
       </c>
       <c r="K61" t="n">
-        <v>-1.556</v>
+        <v>-1.651</v>
       </c>
       <c r="L61" t="n">
-        <v>-6.28</v>
+        <v>-3.7</v>
       </c>
       <c r="M61" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3511,46 +3511,46 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45735</v>
+        <v>45655</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Wailea Golf Club Emerald Course</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E62" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F62" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G62" t="n">
-        <v>1.722</v>
+        <v>1.889</v>
       </c>
       <c r="H62" t="n">
-        <v>0.556</v>
+        <v>0.333</v>
       </c>
       <c r="I62" t="n">
-        <v>0.5</v>
+        <v>0.786</v>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="K62" t="n">
-        <v>-0.676</v>
+        <v>-1.556</v>
       </c>
       <c r="L62" t="n">
-        <v>-1.6</v>
+        <v>-6.28</v>
       </c>
       <c r="M62" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3561,46 +3561,46 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>45829</v>
+        <v>45735</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E63" t="n">
+        <v>10</v>
+      </c>
+      <c r="F63" t="n">
         <v>7</v>
       </c>
-      <c r="F63" t="n">
-        <v>9</v>
-      </c>
       <c r="G63" t="n">
-        <v>1.556</v>
+        <v>1.722</v>
       </c>
       <c r="H63" t="n">
-        <v>0.389</v>
+        <v>0.556</v>
       </c>
       <c r="I63" t="n">
-        <v>0.643</v>
+        <v>0.5</v>
       </c>
       <c r="J63" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="K63" t="n">
-        <v>-1.45</v>
+        <v>-0.676</v>
       </c>
       <c r="L63" t="n">
-        <v>0.14</v>
+        <v>-1.6</v>
       </c>
       <c r="M63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3611,46 +3611,46 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45831</v>
+        <v>45829</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E64" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F64" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G64" t="n">
-        <v>1.778</v>
+        <v>1.556</v>
       </c>
       <c r="H64" t="n">
-        <v>0.444</v>
+        <v>0.389</v>
       </c>
       <c r="I64" t="n">
-        <v>0.571</v>
+        <v>0.643</v>
       </c>
       <c r="J64" t="n">
-        <v>0.3</v>
+        <v>0.45</v>
       </c>
       <c r="K64" t="n">
-        <v>0.247</v>
+        <v>-1.45</v>
       </c>
       <c r="L64" t="n">
-        <v>-3.02</v>
+        <v>0.14</v>
       </c>
       <c r="M64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3661,11 +3661,11 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>45844</v>
+        <v>45831</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3675,7 +3675,7 @@
         <v>8</v>
       </c>
       <c r="F65" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G65" t="n">
         <v>1.778</v>
@@ -3684,23 +3684,23 @@
         <v>0.444</v>
       </c>
       <c r="I65" t="n">
-        <v>0.5</v>
+        <v>0.571</v>
       </c>
       <c r="J65" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="K65" t="n">
-        <v>-1.596</v>
+        <v>0.247</v>
       </c>
       <c r="L65" t="n">
-        <v>-3.44</v>
+        <v>-3.02</v>
       </c>
       <c r="M65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>45857</v>
+        <v>45844</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -3719,38 +3719,38 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E66" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F66" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G66" t="n">
-        <v>1.833</v>
+        <v>1.778</v>
       </c>
       <c r="H66" t="n">
-        <v>0.611</v>
+        <v>0.444</v>
       </c>
       <c r="I66" t="n">
-        <v>0.571</v>
+        <v>0.5</v>
       </c>
       <c r="J66" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="K66" t="n">
-        <v>0.904</v>
+        <v>-1.596</v>
       </c>
       <c r="L66" t="n">
-        <v>-3.18</v>
+        <v>-3.44</v>
       </c>
       <c r="M66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>Fairway Putter</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -3761,39 +3761,39 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>45868</v>
+        <v>45857</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Bethpage Red</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E67" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F67" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G67" t="n">
-        <v>1.611</v>
+        <v>1.833</v>
       </c>
       <c r="H67" t="n">
-        <v>0.222</v>
+        <v>0.611</v>
       </c>
       <c r="I67" t="n">
-        <v>0.5</v>
+        <v>0.571</v>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K67" t="n">
-        <v>-1.342</v>
+        <v>0.904</v>
       </c>
       <c r="L67" t="n">
-        <v>-2.12</v>
+        <v>-3.18</v>
       </c>
       <c r="M67" t="n">
         <v>2</v>
@@ -3811,46 +3811,46 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>45886</v>
+        <v>45868</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Spring Lake Thunderbird</t>
+          <t>Bethpage Red</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E68" t="n">
         <v>4</v>
       </c>
       <c r="F68" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G68" t="n">
-        <v>1.667</v>
+        <v>1.611</v>
       </c>
       <c r="H68" t="n">
         <v>0.222</v>
       </c>
       <c r="I68" t="n">
-        <v>0.786</v>
+        <v>0.5</v>
       </c>
       <c r="J68" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="K68" t="n">
-        <v>-3.573</v>
+        <v>-1.342</v>
       </c>
       <c r="L68" t="n">
-        <v>-3.12</v>
+        <v>-2.12</v>
       </c>
       <c r="M68" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>45892</v>
+        <v>45886</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -3869,38 +3869,38 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E69" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F69" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G69" t="n">
-        <v>1.778</v>
+        <v>1.667</v>
       </c>
       <c r="H69" t="n">
-        <v>0.278</v>
+        <v>0.222</v>
       </c>
       <c r="I69" t="n">
-        <v>0.429</v>
+        <v>0.786</v>
       </c>
       <c r="J69" t="n">
-        <v>-0.3</v>
+        <v>1.2</v>
       </c>
       <c r="K69" t="n">
-        <v>-3.153</v>
+        <v>-3.573</v>
       </c>
       <c r="L69" t="n">
-        <v>-4.7</v>
+        <v>-3.12</v>
       </c>
       <c r="M69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>Greenskeeper</t>
+          <t>Ball Striker</t>
         </is>
       </c>
     </row>
@@ -3911,42 +3911,42 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>45894</v>
+        <v>45892</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Willow Creek Hamlet Course</t>
+          <t>Spring Lake Thunderbird</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E70" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F70" t="n">
         <v>6</v>
       </c>
       <c r="G70" t="n">
-        <v>2.111</v>
+        <v>1.778</v>
       </c>
       <c r="H70" t="n">
-        <v>0.056</v>
+        <v>0.278</v>
       </c>
       <c r="I70" t="n">
         <v>0.429</v>
       </c>
       <c r="J70" t="n">
-        <v>-0.15</v>
+        <v>-0.3</v>
       </c>
       <c r="K70" t="n">
-        <v>-5.517</v>
+        <v>-3.153</v>
       </c>
       <c r="L70" t="n">
-        <v>-12.38</v>
+        <v>-4.7</v>
       </c>
       <c r="M70" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
@@ -3961,46 +3961,46 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>45897</v>
+        <v>45894</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Spring Lake Thunderbird</t>
+          <t>Willow Creek Hamlet Course</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E71" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F71" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G71" t="n">
-        <v>1.722</v>
+        <v>2.111</v>
       </c>
       <c r="H71" t="n">
-        <v>0.222</v>
+        <v>0.056</v>
       </c>
       <c r="I71" t="n">
-        <v>0.214</v>
+        <v>0.429</v>
       </c>
       <c r="J71" t="n">
-        <v>-1.2</v>
+        <v>-0.15</v>
       </c>
       <c r="K71" t="n">
-        <v>-5.733</v>
+        <v>-5.517</v>
       </c>
       <c r="L71" t="n">
-        <v>-4.12</v>
+        <v>-12.38</v>
       </c>
       <c r="M71" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>All Average</t>
         </is>
       </c>
     </row>
@@ -4011,27 +4011,27 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>45941</v>
+        <v>45897</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Wind Watch Hamlet Course</t>
+          <t>Spring Lake Thunderbird</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E72" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F72" t="n">
         <v>3</v>
       </c>
       <c r="G72" t="n">
-        <v>1.667</v>
+        <v>1.722</v>
       </c>
       <c r="H72" t="n">
-        <v>0.056</v>
+        <v>0.222</v>
       </c>
       <c r="I72" t="n">
         <v>0.214</v>
@@ -4040,17 +4040,17 @@
         <v>-1.2</v>
       </c>
       <c r="K72" t="n">
-        <v>-5.522</v>
+        <v>-5.733</v>
       </c>
       <c r="L72" t="n">
-        <v>-4.38</v>
+        <v>-4.12</v>
       </c>
       <c r="M72" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>Ball Striker</t>
+          <t>Fairway Putter</t>
         </is>
       </c>
     </row>
@@ -4061,39 +4061,39 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>46160</v>
+        <v>45941</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Bethpage Blue</t>
+          <t>Wind Watch Hamlet Course</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E73" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F73" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G73" t="n">
-        <v>1.889</v>
+        <v>1.667</v>
       </c>
       <c r="H73" t="n">
-        <v>0.444</v>
+        <v>0.056</v>
       </c>
       <c r="I73" t="n">
-        <v>0.357</v>
+        <v>0.214</v>
       </c>
       <c r="J73" t="n">
-        <v>-0.6</v>
+        <v>-1.2</v>
       </c>
       <c r="K73" t="n">
-        <v>-0.173</v>
+        <v>-5.522</v>
       </c>
       <c r="L73" t="n">
-        <v>-5.44</v>
+        <v>-4.38</v>
       </c>
       <c r="M73" t="n">
         <v>3</v>
@@ -4111,46 +4111,46 @@
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>46164</v>
+        <v>46160</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Brentwood Country Club</t>
+          <t>Bethpage Blue</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E74" t="n">
+        <v>8</v>
+      </c>
+      <c r="F74" t="n">
+        <v>5</v>
+      </c>
+      <c r="G74" t="n">
+        <v>1.889</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="I74" t="n">
+        <v>0.357</v>
+      </c>
+      <c r="J74" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="K74" t="n">
+        <v>-0.173</v>
+      </c>
+      <c r="L74" t="n">
+        <v>-5.44</v>
+      </c>
+      <c r="M74" t="n">
         <v>2</v>
       </c>
-      <c r="F74" t="n">
-        <v>9</v>
-      </c>
-      <c r="G74" t="n">
-        <v>1.722</v>
-      </c>
-      <c r="H74" t="n">
-        <v>0.111</v>
-      </c>
-      <c r="I74" t="n">
-        <v>0.643</v>
-      </c>
-      <c r="J74" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="K74" t="n">
-        <v>-3.95</v>
-      </c>
-      <c r="L74" t="n">
-        <v>-4.96</v>
-      </c>
-      <c r="M74" t="n">
-        <v>0</v>
-      </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>All Average</t>
+          <t>Greenskeeper</t>
         </is>
       </c>
     </row>
@@ -4161,39 +4161,39 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>46173</v>
+        <v>46164</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Bethpage Green</t>
+          <t>Brentwood Country Club</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E75" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F75" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G75" t="n">
-        <v>1.944</v>
+        <v>1.722</v>
       </c>
       <c r="H75" t="n">
-        <v>0.278</v>
+        <v>0.111</v>
       </c>
       <c r="I75" t="n">
-        <v>0.357</v>
+        <v>0.643</v>
       </c>
       <c r="J75" t="n">
-        <v>-0.6</v>
+        <v>0.45</v>
       </c>
       <c r="K75" t="n">
-        <v>-3.256</v>
+        <v>-3.95</v>
       </c>
       <c r="L75" t="n">
-        <v>-7.7</v>
+        <v>-4.96</v>
       </c>
       <c r="M75" t="n">
         <v>1</v>
@@ -4211,11 +4211,11 @@
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>46201</v>
+        <v>46173</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Spring Lake Thunderbird</t>
+          <t>Bethpage Green</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4225,7 +4225,7 @@
         <v>5</v>
       </c>
       <c r="F76" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G76" t="n">
         <v>1.944</v>
@@ -4234,21 +4234,121 @@
         <v>0.278</v>
       </c>
       <c r="I76" t="n">
-        <v>0.429</v>
+        <v>0.357</v>
       </c>
       <c r="J76" t="n">
-        <v>-0.3</v>
+        <v>-0.6</v>
       </c>
       <c r="K76" t="n">
-        <v>-2.722</v>
+        <v>-3.256</v>
       </c>
       <c r="L76" t="n">
         <v>-7.7</v>
       </c>
       <c r="M76" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>All Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>46201</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Spring Lake Thunderbird</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>35</v>
+      </c>
+      <c r="E77" t="n">
+        <v>5</v>
+      </c>
+      <c r="F77" t="n">
+        <v>6</v>
+      </c>
+      <c r="G77" t="n">
+        <v>1.944</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="J77" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="K77" t="n">
+        <v>-2.722</v>
+      </c>
+      <c r="L77" t="n">
+        <v>-7.7</v>
+      </c>
+      <c r="M77" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>All Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Brentwood Country Club</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>29</v>
+      </c>
+      <c r="E78" t="n">
+        <v>6</v>
+      </c>
+      <c r="F78" t="n">
+        <v>11</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1.611</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0.786</v>
+      </c>
+      <c r="J78" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="K78" t="n">
+        <v>-4.95</v>
+      </c>
+      <c r="L78" t="n">
+        <v>-1.28</v>
+      </c>
+      <c r="M78" t="n">
         <v>1</v>
       </c>
-      <c r="N76" t="inlineStr">
+      <c r="N78" t="inlineStr">
         <is>
           <t>Ball Striker</t>
         </is>

</xml_diff>